<commit_message>
Actualiza diccionario CECOS (estructura nueva)
- CECOS.xlsx actualizado (reasignaciones de VP/Gerencia).
- Regenerados v3, BBDD (dim_cecos) y los dashboards + Excel por VP.
- La VP "Otros - Arriendos" ya no tiene CECOs propios en la estructura nueva: se elimina
  su dashboard (sus CECOs pasaron a otras VPs; totales sin cambio).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCAC711-D6A2-4D3D-A1DB-EFDE555B5AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378D13A9-4301-431E-BAD4-21816CF5DD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -9329,7 +9329,7 @@
     <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -9398,6 +9398,9 @@
     <xf numFmtId="0" fontId="15" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="63">
@@ -65667,7 +65670,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:P308"/>
@@ -65740,7 +65743,7 @@
         <v>2312</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2313</v>
       </c>
@@ -65787,7 +65790,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2313</v>
       </c>
@@ -65834,7 +65837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2313</v>
       </c>
@@ -65881,7 +65884,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2313</v>
       </c>
@@ -65928,7 +65931,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2313</v>
       </c>
@@ -65975,7 +65978,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2313</v>
       </c>
@@ -66022,7 +66025,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2313</v>
       </c>
@@ -66069,7 +66072,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2313</v>
       </c>
@@ -66116,7 +66119,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2313</v>
       </c>
@@ -66163,7 +66166,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2313</v>
       </c>
@@ -66210,7 +66213,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>2313</v>
       </c>
@@ -66260,7 +66263,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2313</v>
       </c>
@@ -66308,7 +66311,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>2313</v>
       </c>
@@ -66355,7 +66358,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2313</v>
       </c>
@@ -66402,7 +66405,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>2313</v>
       </c>
@@ -66449,7 +66452,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2313</v>
       </c>
@@ -66496,7 +66499,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2313</v>
       </c>
@@ -66543,7 +66546,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>2313</v>
       </c>
@@ -66590,7 +66593,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2313</v>
       </c>
@@ -66637,7 +66640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>2313</v>
       </c>
@@ -66687,7 +66690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>2313</v>
       </c>
@@ -66734,7 +66737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2313</v>
       </c>
@@ -66781,7 +66784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2313</v>
       </c>
@@ -66828,7 +66831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2313</v>
       </c>
@@ -66875,7 +66878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2313</v>
       </c>
@@ -66922,7 +66925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>2313</v>
       </c>
@@ -66969,7 +66972,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2313</v>
       </c>
@@ -67019,7 +67022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2313</v>
       </c>
@@ -67066,7 +67069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2313</v>
       </c>
@@ -67113,7 +67116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>2313</v>
       </c>
@@ -67160,7 +67163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2313</v>
       </c>
@@ -68109,7 +68112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>2313</v>
       </c>
@@ -68156,7 +68159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>2313</v>
       </c>
@@ -68203,7 +68206,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>2313</v>
       </c>
@@ -68250,7 +68253,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>2313</v>
       </c>
@@ -68297,7 +68300,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>2313</v>
       </c>
@@ -68344,7 +68347,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>2313</v>
       </c>
@@ -68391,7 +68394,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>2313</v>
       </c>
@@ -68438,7 +68441,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>2313</v>
       </c>
@@ -68485,7 +68488,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>2313</v>
       </c>
@@ -68532,7 +68535,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>2313</v>
       </c>
@@ -68579,7 +68582,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>2313</v>
       </c>
@@ -68626,7 +68629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>2313</v>
       </c>
@@ -68673,7 +68676,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>2313</v>
       </c>
@@ -68720,7 +68723,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>2313</v>
       </c>
@@ -68767,7 +68770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>2313</v>
       </c>
@@ -68814,7 +68817,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>2313</v>
       </c>
@@ -68864,7 +68867,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>2313</v>
       </c>
@@ -68911,7 +68914,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>2313</v>
       </c>
@@ -68958,7 +68961,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>2313</v>
       </c>
@@ -69005,7 +69008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>2313</v>
       </c>
@@ -69055,7 +69058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>2313</v>
       </c>
@@ -69102,7 +69105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>2313</v>
       </c>
@@ -69149,7 +69152,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>2313</v>
       </c>
@@ -69199,7 +69202,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>2313</v>
       </c>
@@ -69247,7 +69250,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>2313</v>
       </c>
@@ -69294,7 +69297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>2313</v>
       </c>
@@ -69344,7 +69347,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>2313</v>
       </c>
@@ -69391,7 +69394,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>2313</v>
       </c>
@@ -69438,7 +69441,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>2313</v>
       </c>
@@ -69485,7 +69488,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>2313</v>
       </c>
@@ -69535,7 +69538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>2313</v>
       </c>
@@ -69585,7 +69588,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>2313</v>
       </c>
@@ -69632,7 +69635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>2313</v>
       </c>
@@ -69679,7 +69682,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>2313</v>
       </c>
@@ -69726,7 +69729,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>2313</v>
       </c>
@@ -69773,7 +69776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>2313</v>
       </c>
@@ -69820,7 +69823,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>2313</v>
       </c>
@@ -69867,7 +69870,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>2313</v>
       </c>
@@ -69915,7 +69918,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>2313</v>
       </c>
@@ -69963,7 +69966,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>2313</v>
       </c>
@@ -70010,7 +70013,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>2313</v>
       </c>
@@ -70057,7 +70060,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>2313</v>
       </c>
@@ -70104,7 +70107,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>2313</v>
       </c>
@@ -70151,7 +70154,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>2313</v>
       </c>
@@ -70198,7 +70201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>2313</v>
       </c>
@@ -70245,7 +70248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>2313</v>
       </c>
@@ -70292,7 +70295,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>2313</v>
       </c>
@@ -70339,7 +70342,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>2313</v>
       </c>
@@ -70386,7 +70389,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>2313</v>
       </c>
@@ -70433,7 +70436,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>2313</v>
       </c>
@@ -70480,7 +70483,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>2313</v>
       </c>
@@ -70527,7 +70530,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>2313</v>
       </c>
@@ -70574,7 +70577,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>2313</v>
       </c>
@@ -70621,7 +70624,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>2313</v>
       </c>
@@ -70668,7 +70671,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>2313</v>
       </c>
@@ -70715,7 +70718,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>2313</v>
       </c>
@@ -70765,7 +70768,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>2313</v>
       </c>
@@ -70812,7 +70815,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>2313</v>
       </c>
@@ -70859,7 +70862,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>2313</v>
       </c>
@@ -70906,7 +70909,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>2313</v>
       </c>
@@ -70953,7 +70956,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>2313</v>
       </c>
@@ -71000,7 +71003,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>2313</v>
       </c>
@@ -71047,7 +71050,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>2313</v>
       </c>
@@ -71094,7 +71097,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>2313</v>
       </c>
@@ -71141,7 +71144,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>2313</v>
       </c>
@@ -71188,7 +71191,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>2313</v>
       </c>
@@ -71235,7 +71238,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>2313</v>
       </c>
@@ -71282,7 +71285,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>2313</v>
       </c>
@@ -71329,7 +71332,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>2313</v>
       </c>
@@ -71376,7 +71379,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>2313</v>
       </c>
@@ -71423,7 +71426,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>2313</v>
       </c>
@@ -71470,7 +71473,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>2313</v>
       </c>
@@ -71520,7 +71523,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>2313</v>
       </c>
@@ -71567,7 +71570,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>2313</v>
       </c>
@@ -71617,7 +71620,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>2313</v>
       </c>
@@ -71664,7 +71667,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>2313</v>
       </c>
@@ -71714,7 +71717,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>2313</v>
       </c>
@@ -71761,7 +71764,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71808,7 +71811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71855,7 +71858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2313</v>
       </c>
@@ -71902,7 +71905,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>2313</v>
       </c>
@@ -71949,7 +71952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>2313</v>
       </c>
@@ -71996,7 +71999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>2313</v>
       </c>
@@ -72043,7 +72046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>2313</v>
       </c>
@@ -72090,7 +72093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>2313</v>
       </c>
@@ -72140,7 +72143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>2313</v>
       </c>
@@ -72187,7 +72190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72234,7 +72237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>2313</v>
       </c>
@@ -72281,7 +72284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>2313</v>
       </c>
@@ -72328,7 +72331,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>2313</v>
       </c>
@@ -72469,7 +72472,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>2313</v>
       </c>
@@ -72516,7 +72519,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>2313</v>
       </c>
@@ -72563,7 +72566,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>2313</v>
       </c>
@@ -72610,7 +72613,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72657,7 +72660,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72704,7 +72707,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>2313</v>
       </c>
@@ -72751,7 +72754,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>2313</v>
       </c>
@@ -72798,7 +72801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>2313</v>
       </c>
@@ -72845,7 +72848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>2313</v>
       </c>
@@ -72895,7 +72898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>2313</v>
       </c>
@@ -72942,7 +72945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>2313</v>
       </c>
@@ -72989,7 +72992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73036,7 +73039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>2313</v>
       </c>
@@ -73083,7 +73086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>2313</v>
       </c>
@@ -73130,7 +73133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>2313</v>
       </c>
@@ -73177,7 +73180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>2313</v>
       </c>
@@ -73224,7 +73227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>2313</v>
       </c>
@@ -73365,7 +73368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>2313</v>
       </c>
@@ -73412,7 +73415,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>2313</v>
       </c>
@@ -73459,7 +73462,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73506,7 +73509,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73553,7 +73556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>2313</v>
       </c>
@@ -73600,7 +73603,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>2313</v>
       </c>
@@ -73647,7 +73650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>2313</v>
       </c>
@@ -73694,7 +73697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>2313</v>
       </c>
@@ -73741,7 +73744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73788,7 +73791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>2313</v>
       </c>
@@ -73835,7 +73838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>2313</v>
       </c>
@@ -73885,7 +73888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>2313</v>
       </c>
@@ -73932,7 +73935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>2313</v>
       </c>
@@ -74026,7 +74029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>2313</v>
       </c>
@@ -74120,7 +74123,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>2313</v>
       </c>
@@ -74167,7 +74170,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>2313</v>
       </c>
@@ -74214,7 +74217,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>2313</v>
       </c>
@@ -74261,7 +74264,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>2313</v>
       </c>
@@ -74308,7 +74311,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="183" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74355,7 +74358,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74402,7 +74405,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>2313</v>
       </c>
@@ -74449,7 +74452,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>2313</v>
       </c>
@@ -74496,7 +74499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>2313</v>
       </c>
@@ -74543,7 +74546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>2313</v>
       </c>
@@ -74590,7 +74593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>2313</v>
       </c>
@@ -74640,7 +74643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>2313</v>
       </c>
@@ -74687,7 +74690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74734,7 +74737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>2313</v>
       </c>
@@ -74781,7 +74784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>2313</v>
       </c>
@@ -74922,7 +74925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>2313</v>
       </c>
@@ -74969,7 +74972,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>2313</v>
       </c>
@@ -75016,7 +75019,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>2313</v>
       </c>
@@ -75063,7 +75066,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>2313</v>
       </c>
@@ -75110,7 +75113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>2313</v>
       </c>
@@ -75157,7 +75160,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>2313</v>
       </c>
@@ -75204,7 +75207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>2313</v>
       </c>
@@ -75254,7 +75257,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="203" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75301,7 +75304,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="204" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75348,7 +75351,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="205" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75395,7 +75398,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>2313</v>
       </c>
@@ -75443,7 +75446,7 @@
       </c>
       <c r="P206" s="3"/>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>2313</v>
       </c>
@@ -75491,7 +75494,7 @@
       </c>
       <c r="P207" s="3"/>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>2313</v>
       </c>
@@ -75539,7 +75542,7 @@
       </c>
       <c r="P208" s="3"/>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>2313</v>
       </c>
@@ -75587,7 +75590,7 @@
       </c>
       <c r="P209" s="3"/>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>2313</v>
       </c>
@@ -75635,7 +75638,7 @@
       </c>
       <c r="P210" s="3"/>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>2313</v>
       </c>
@@ -75683,7 +75686,7 @@
       </c>
       <c r="P211" s="3"/>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>2313</v>
       </c>
@@ -75731,7 +75734,7 @@
       </c>
       <c r="P212" s="3"/>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>2313</v>
       </c>
@@ -75779,7 +75782,7 @@
       </c>
       <c r="P213" s="3"/>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>2313</v>
       </c>
@@ -75827,7 +75830,7 @@
       </c>
       <c r="P214" s="3"/>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>2313</v>
       </c>
@@ -75875,7 +75878,7 @@
       </c>
       <c r="P215" s="3"/>
     </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>2313</v>
       </c>
@@ -75923,7 +75926,7 @@
       </c>
       <c r="P216" s="3"/>
     </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>2313</v>
       </c>
@@ -75970,7 +75973,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>2313</v>
       </c>
@@ -76017,7 +76020,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>2313</v>
       </c>
@@ -76064,7 +76067,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>2313</v>
       </c>
@@ -76111,7 +76114,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>2313</v>
       </c>
@@ -76158,7 +76161,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>2313</v>
       </c>
@@ -76205,7 +76208,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>2313</v>
       </c>
@@ -76252,7 +76255,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>2313</v>
       </c>
@@ -76299,7 +76302,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>2313</v>
       </c>
@@ -76346,7 +76349,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>2313</v>
       </c>
@@ -76393,7 +76396,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>2313</v>
       </c>
@@ -76440,7 +76443,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>2313</v>
       </c>
@@ -76487,7 +76490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>2313</v>
       </c>
@@ -76534,7 +76537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>2313</v>
       </c>
@@ -76581,7 +76584,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>2313</v>
       </c>
@@ -76628,7 +76631,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>2685</v>
       </c>
@@ -76675,7 +76678,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>2654</v>
       </c>
@@ -76720,52 +76723,54 @@
       </c>
       <c r="P233" s="3"/>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
+        <v>2313</v>
+      </c>
+      <c r="B234" t="s">
+        <v>664</v>
+      </c>
+      <c r="C234" t="s">
+        <v>2314</v>
+      </c>
+      <c r="D234" s="31" t="s">
+        <v>2741</v>
+      </c>
+      <c r="E234" s="27" t="s">
         <v>2740</v>
       </c>
-      <c r="B234" t="s">
+      <c r="F234" s="27" t="s">
         <v>2740</v>
       </c>
-      <c r="C234" t="s">
-        <v>2740</v>
-      </c>
-      <c r="D234" s="6" t="s">
-        <v>2741</v>
-      </c>
-      <c r="E234" t="s">
-        <v>2740</v>
-      </c>
-      <c r="F234" t="s">
-        <v>2740</v>
-      </c>
       <c r="G234" t="s">
-        <v>2742</v>
+        <v>2317</v>
       </c>
       <c r="H234" t="s">
-        <v>2743</v>
+        <v>2318</v>
       </c>
       <c r="I234" t="s">
-        <v>2744</v>
+        <v>2413</v>
       </c>
       <c r="J234" t="s">
-        <v>2745</v>
-      </c>
-      <c r="K234" s="6" t="s">
-        <v>2741</v>
+        <v>2414</v>
+      </c>
+      <c r="K234" t="s">
+        <v>2413</v>
       </c>
       <c r="L234" t="s">
-        <v>2740</v>
+        <v>2414</v>
       </c>
       <c r="M234" t="s">
-        <v>2682</v>
-      </c>
-      <c r="O234" s="17" t="s">
-        <v>2321</v>
-      </c>
-      <c r="P234" s="3"/>
-    </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.3">
+        <v>2415</v>
+      </c>
+      <c r="O234" s="28" t="s">
+        <v>2583</v>
+      </c>
+      <c r="P234" s="28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>2685</v>
       </c>
@@ -76812,7 +76817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>2685</v>
       </c>
@@ -76859,7 +76864,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>2685</v>
       </c>
@@ -76906,7 +76911,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>2685</v>
       </c>
@@ -76953,7 +76958,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>2685</v>
       </c>
@@ -77000,7 +77005,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>2685</v>
       </c>
@@ -77047,7 +77052,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>2685</v>
       </c>
@@ -77094,7 +77099,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>2313</v>
       </c>
@@ -77141,7 +77146,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>2313</v>
       </c>
@@ -77188,7 +77193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>2313</v>
       </c>
@@ -77235,7 +77240,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>2313</v>
       </c>
@@ -77282,7 +77287,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>2313</v>
       </c>
@@ -77329,7 +77334,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>2313</v>
       </c>
@@ -77376,7 +77381,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>2313</v>
       </c>
@@ -77423,7 +77428,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>2313</v>
       </c>
@@ -77470,7 +77475,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>2313</v>
       </c>
@@ -77517,7 +77522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>2313</v>
       </c>
@@ -77564,7 +77569,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>2313</v>
       </c>
@@ -77611,7 +77616,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>2313</v>
       </c>
@@ -77658,7 +77663,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>2313</v>
       </c>
@@ -77705,7 +77710,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>2313</v>
       </c>
@@ -77752,7 +77757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>2313</v>
       </c>
@@ -77799,7 +77804,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="257" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>2313</v>
       </c>
@@ -77846,7 +77851,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="258" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" s="13" t="s">
         <v>2313</v>
       </c>
@@ -77893,7 +77898,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2313</v>
       </c>
@@ -77940,7 +77945,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="260" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2313</v>
       </c>
@@ -77987,7 +77992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2313</v>
       </c>
@@ -78034,7 +78039,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2313</v>
       </c>
@@ -78081,7 +78086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2313</v>
       </c>
@@ -78128,7 +78133,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2313</v>
       </c>
@@ -78175,7 +78180,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2313</v>
       </c>
@@ -78222,7 +78227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78269,7 +78274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78316,7 +78321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78363,7 +78368,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78410,7 +78415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78457,7 +78462,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78504,7 +78509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78545,7 +78550,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="273" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78586,7 +78591,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="274" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78633,7 +78638,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78680,7 +78685,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="276" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78727,7 +78732,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78771,7 +78776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="11" t="s">
         <v>2313</v>
       </c>
@@ -79946,7 +79951,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2313</v>
       </c>
@@ -79993,7 +79998,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2313</v>
       </c>
@@ -80040,7 +80045,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2313</v>
       </c>
@@ -80087,7 +80092,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="306" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2313</v>
       </c>
@@ -80134,7 +80139,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2313</v>
       </c>
@@ -80181,7 +80186,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="308" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2313</v>
       </c>
@@ -80229,7 +80234,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}"/>
+  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
+    <filterColumn colId="12">
+      <filters>
+        <filter val="VPPyO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="D278 D1:D271">
     <cfRule type="duplicateValues" dxfId="10" priority="1"/>
     <cfRule type="duplicateValues" dxfId="9" priority="11"/>
@@ -80270,12 +80281,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="70b3a8a4-10f1-4453-b557-059c8aa2e01d" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -80540,21 +80554,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="70b3a8a4-10f1-4453-b557-059c8aa2e01d" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
+    <ds:schemaRef ds:uri="70b3a8a4-10f1-4453-b557-059c8aa2e01d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -80579,12 +80593,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
-    <ds:schemaRef ds:uri="70b3a8a4-10f1-4453-b557-059c8aa2e01d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualiza Ppto 2027 (PPTO27_13_07_2026_15_30) y CECOS
- Nuevo Ppto: PPTO27_13_07_2026_15_30.XLSX (4191 filas). Total Ppto 2027: 475,893 MM
  (antes 290,403 · +185 MM, Ppto mas completo). Reemplaza el 13_07 (borrado).
- CECOS.xlsx actualizado.
- Regenerados v3 (con el boton toggle ya commiteado), BBDD y 23 dashboards + Excel por VP.
  Corrige el v3 del commit anterior (a7eb9ae), que habia quedado con Ppto 2027 = 0 porque
  el archivo de Ppto se borro durante ese build.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378D13A9-4301-431E-BAD4-21816CF5DD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEB9DDA-6561-403F-8535-933A644FCF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19682" uniqueCount="2900">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19682" uniqueCount="2907">
   <si>
     <t>Clasificación 1</t>
   </si>
@@ -8745,6 +8745,27 @@
   </si>
   <si>
     <t>N1005AD5504</t>
+  </si>
+  <si>
+    <t>Compliance AMSA</t>
+  </si>
+  <si>
+    <t>Compliance MLP</t>
+  </si>
+  <si>
+    <t>Propiedad Minera CEN</t>
+  </si>
+  <si>
+    <t>Compliance CEN</t>
+  </si>
+  <si>
+    <t>Propiedad Minera ANT</t>
+  </si>
+  <si>
+    <t>Compliance ANT</t>
+  </si>
+  <si>
+    <t>Compliance CMZ</t>
   </si>
 </sst>
 </file>
@@ -65670,7 +65691,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:P308"/>
@@ -65743,7 +65764,7 @@
         <v>2312</v>
       </c>
     </row>
-    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2313</v>
       </c>
@@ -65790,7 +65811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2313</v>
       </c>
@@ -65837,7 +65858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2313</v>
       </c>
@@ -65884,7 +65905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2313</v>
       </c>
@@ -65931,7 +65952,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2313</v>
       </c>
@@ -65978,7 +65999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2313</v>
       </c>
@@ -66025,7 +66046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2313</v>
       </c>
@@ -66072,7 +66093,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2313</v>
       </c>
@@ -66119,7 +66140,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2313</v>
       </c>
@@ -66166,7 +66187,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2313</v>
       </c>
@@ -66213,7 +66234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>2313</v>
       </c>
@@ -66263,7 +66284,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2313</v>
       </c>
@@ -66311,7 +66332,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>2313</v>
       </c>
@@ -66358,7 +66379,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2313</v>
       </c>
@@ -66405,7 +66426,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>2313</v>
       </c>
@@ -66452,7 +66473,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2313</v>
       </c>
@@ -66499,7 +66520,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2313</v>
       </c>
@@ -66546,7 +66567,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>2313</v>
       </c>
@@ -66593,7 +66614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2313</v>
       </c>
@@ -66640,7 +66661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>2313</v>
       </c>
@@ -66690,7 +66711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>2313</v>
       </c>
@@ -66737,7 +66758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2313</v>
       </c>
@@ -66784,7 +66805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2313</v>
       </c>
@@ -66831,7 +66852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2313</v>
       </c>
@@ -66878,7 +66899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2313</v>
       </c>
@@ -66925,7 +66946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>2313</v>
       </c>
@@ -66972,7 +66993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2313</v>
       </c>
@@ -67022,7 +67043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2313</v>
       </c>
@@ -67069,7 +67090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2313</v>
       </c>
@@ -67116,7 +67137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>2313</v>
       </c>
@@ -67163,7 +67184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2313</v>
       </c>
@@ -68112,7 +68133,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>2313</v>
       </c>
@@ -68159,7 +68180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>2313</v>
       </c>
@@ -68206,7 +68227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>2313</v>
       </c>
@@ -68253,7 +68274,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>2313</v>
       </c>
@@ -68300,7 +68321,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>2313</v>
       </c>
@@ -68347,7 +68368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>2313</v>
       </c>
@@ -68394,7 +68415,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>2313</v>
       </c>
@@ -68441,7 +68462,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>2313</v>
       </c>
@@ -68488,7 +68509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>2313</v>
       </c>
@@ -68535,7 +68556,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>2313</v>
       </c>
@@ -68570,7 +68591,7 @@
         <v>2478</v>
       </c>
       <c r="L61" t="s">
-        <v>2477</v>
+        <v>2669</v>
       </c>
       <c r="M61" t="s">
         <v>2479</v>
@@ -68582,7 +68603,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>2313</v>
       </c>
@@ -68617,7 +68638,7 @@
         <v>2478</v>
       </c>
       <c r="L62" t="s">
-        <v>2477</v>
+        <v>775</v>
       </c>
       <c r="M62" t="s">
         <v>2479</v>
@@ -68629,7 +68650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>2313</v>
       </c>
@@ -68664,7 +68685,7 @@
         <v>2478</v>
       </c>
       <c r="L63" t="s">
-        <v>2477</v>
+        <v>775</v>
       </c>
       <c r="M63" t="s">
         <v>2479</v>
@@ -68676,7 +68697,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>2313</v>
       </c>
@@ -68690,7 +68711,7 @@
         <v>2855</v>
       </c>
       <c r="E64" s="22" t="s">
-        <v>2856</v>
+        <v>2900</v>
       </c>
       <c r="F64" s="22" t="s">
         <v>2856</v>
@@ -68710,8 +68731,8 @@
       <c r="K64" s="22" t="s">
         <v>2478</v>
       </c>
-      <c r="L64" s="22" t="s">
-        <v>2477</v>
+      <c r="L64" t="s">
+        <v>2856</v>
       </c>
       <c r="M64" s="22" t="s">
         <v>2479</v>
@@ -68723,7 +68744,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>2313</v>
       </c>
@@ -68758,7 +68779,7 @@
         <v>2478</v>
       </c>
       <c r="L65" t="s">
-        <v>2477</v>
+        <v>775</v>
       </c>
       <c r="M65" t="s">
         <v>2479</v>
@@ -68770,7 +68791,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>2313</v>
       </c>
@@ -68817,7 +68838,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>2313</v>
       </c>
@@ -68867,7 +68888,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>2313</v>
       </c>
@@ -68914,7 +68935,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>2313</v>
       </c>
@@ -68961,7 +68982,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>2313</v>
       </c>
@@ -69008,7 +69029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>2313</v>
       </c>
@@ -69058,7 +69079,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>2313</v>
       </c>
@@ -69105,7 +69126,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>2313</v>
       </c>
@@ -69152,7 +69173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>2313</v>
       </c>
@@ -69202,7 +69223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>2313</v>
       </c>
@@ -69250,7 +69271,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>2313</v>
       </c>
@@ -69297,7 +69318,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>2313</v>
       </c>
@@ -69347,7 +69368,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>2313</v>
       </c>
@@ -69394,7 +69415,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>2313</v>
       </c>
@@ -69441,7 +69462,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>2313</v>
       </c>
@@ -69488,7 +69509,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>2313</v>
       </c>
@@ -69538,7 +69559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>2313</v>
       </c>
@@ -69588,7 +69609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>2313</v>
       </c>
@@ -69635,7 +69656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>2313</v>
       </c>
@@ -69682,7 +69703,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>2313</v>
       </c>
@@ -69729,7 +69750,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>2313</v>
       </c>
@@ -69776,7 +69797,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>2313</v>
       </c>
@@ -69823,7 +69844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>2313</v>
       </c>
@@ -69870,7 +69891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>2313</v>
       </c>
@@ -69918,7 +69939,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>2313</v>
       </c>
@@ -69966,7 +69987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>2313</v>
       </c>
@@ -70013,7 +70034,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>2313</v>
       </c>
@@ -70060,7 +70081,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>2313</v>
       </c>
@@ -70107,7 +70128,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>2313</v>
       </c>
@@ -70154,7 +70175,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>2313</v>
       </c>
@@ -70201,7 +70222,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>2313</v>
       </c>
@@ -70248,7 +70269,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>2313</v>
       </c>
@@ -70295,7 +70316,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>2313</v>
       </c>
@@ -70342,7 +70363,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>2313</v>
       </c>
@@ -70389,7 +70410,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>2313</v>
       </c>
@@ -70436,7 +70457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>2313</v>
       </c>
@@ -70483,7 +70504,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>2313</v>
       </c>
@@ -70530,7 +70551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>2313</v>
       </c>
@@ -70577,7 +70598,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>2313</v>
       </c>
@@ -70624,7 +70645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>2313</v>
       </c>
@@ -70671,7 +70692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>2313</v>
       </c>
@@ -70718,7 +70739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>2313</v>
       </c>
@@ -70768,7 +70789,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>2313</v>
       </c>
@@ -70815,7 +70836,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>2313</v>
       </c>
@@ -70862,7 +70883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>2313</v>
       </c>
@@ -70909,7 +70930,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>2313</v>
       </c>
@@ -70956,7 +70977,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>2313</v>
       </c>
@@ -71003,7 +71024,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>2313</v>
       </c>
@@ -71050,7 +71071,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>2313</v>
       </c>
@@ -71097,7 +71118,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>2313</v>
       </c>
@@ -71144,7 +71165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>2313</v>
       </c>
@@ -71191,7 +71212,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>2313</v>
       </c>
@@ -71238,7 +71259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>2313</v>
       </c>
@@ -71285,7 +71306,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>2313</v>
       </c>
@@ -71332,7 +71353,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>2313</v>
       </c>
@@ -71379,7 +71400,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>2313</v>
       </c>
@@ -71426,7 +71447,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>2313</v>
       </c>
@@ -71473,7 +71494,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>2313</v>
       </c>
@@ -71523,7 +71544,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>2313</v>
       </c>
@@ -71570,7 +71591,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>2313</v>
       </c>
@@ -71620,7 +71641,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>2313</v>
       </c>
@@ -71667,7 +71688,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>2313</v>
       </c>
@@ -71717,7 +71738,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>2313</v>
       </c>
@@ -71764,7 +71785,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A129" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71811,7 +71832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A130" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71858,7 +71879,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2313</v>
       </c>
@@ -71905,7 +71926,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>2313</v>
       </c>
@@ -71952,7 +71973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>2313</v>
       </c>
@@ -71999,7 +72020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>2313</v>
       </c>
@@ -72046,7 +72067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>2313</v>
       </c>
@@ -72093,7 +72114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>2313</v>
       </c>
@@ -72143,7 +72164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>2313</v>
       </c>
@@ -72190,7 +72211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A138" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72237,7 +72258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>2313</v>
       </c>
@@ -72284,7 +72305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>2313</v>
       </c>
@@ -72331,7 +72352,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>2313</v>
       </c>
@@ -72472,7 +72493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>2313</v>
       </c>
@@ -72519,7 +72540,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>2313</v>
       </c>
@@ -72566,7 +72587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>2313</v>
       </c>
@@ -72613,7 +72634,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A147" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72660,7 +72681,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A148" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72707,7 +72728,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>2313</v>
       </c>
@@ -72754,7 +72775,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>2313</v>
       </c>
@@ -72801,7 +72822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>2313</v>
       </c>
@@ -72848,7 +72869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>2313</v>
       </c>
@@ -72898,7 +72919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>2313</v>
       </c>
@@ -72945,7 +72966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>2313</v>
       </c>
@@ -72992,7 +73013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A155" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73039,7 +73060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>2313</v>
       </c>
@@ -73086,7 +73107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>2313</v>
       </c>
@@ -73133,7 +73154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>2313</v>
       </c>
@@ -73180,7 +73201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>2313</v>
       </c>
@@ -73227,7 +73248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>2313</v>
       </c>
@@ -73368,7 +73389,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>2313</v>
       </c>
@@ -73415,7 +73436,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>2313</v>
       </c>
@@ -73462,7 +73483,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A165" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73509,7 +73530,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A166" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73556,7 +73577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>2313</v>
       </c>
@@ -73603,7 +73624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>2313</v>
       </c>
@@ -73650,7 +73671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>2313</v>
       </c>
@@ -73697,7 +73718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>2313</v>
       </c>
@@ -73744,7 +73765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A171" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73791,7 +73812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>2313</v>
       </c>
@@ -73838,7 +73859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>2313</v>
       </c>
@@ -73888,7 +73909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>2313</v>
       </c>
@@ -73935,7 +73956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>2313</v>
       </c>
@@ -74029,7 +74050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>2313</v>
       </c>
@@ -74123,7 +74144,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>2313</v>
       </c>
@@ -74170,7 +74191,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>2313</v>
       </c>
@@ -74217,7 +74238,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>2313</v>
       </c>
@@ -74264,7 +74285,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>2313</v>
       </c>
@@ -74311,7 +74332,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="183" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A183" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74358,7 +74379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A184" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74405,7 +74426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>2313</v>
       </c>
@@ -74452,7 +74473,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>2313</v>
       </c>
@@ -74499,7 +74520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>2313</v>
       </c>
@@ -74546,7 +74567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>2313</v>
       </c>
@@ -74593,7 +74614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>2313</v>
       </c>
@@ -74643,7 +74664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>2313</v>
       </c>
@@ -74690,7 +74711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A191" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74737,7 +74758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>2313</v>
       </c>
@@ -74784,7 +74805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>2313</v>
       </c>
@@ -74925,7 +74946,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>2313</v>
       </c>
@@ -74972,7 +74993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>2313</v>
       </c>
@@ -75019,7 +75040,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>2313</v>
       </c>
@@ -75066,7 +75087,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>2313</v>
       </c>
@@ -75113,7 +75134,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>2313</v>
       </c>
@@ -75160,7 +75181,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>2313</v>
       </c>
@@ -75207,7 +75228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>2313</v>
       </c>
@@ -75257,7 +75278,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="203" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A203" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75304,7 +75325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="204" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A204" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75351,7 +75372,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="205" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A205" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75398,7 +75419,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>2313</v>
       </c>
@@ -75446,7 +75467,7 @@
       </c>
       <c r="P206" s="3"/>
     </row>
-    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>2313</v>
       </c>
@@ -75494,7 +75515,7 @@
       </c>
       <c r="P207" s="3"/>
     </row>
-    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>2313</v>
       </c>
@@ -75542,7 +75563,7 @@
       </c>
       <c r="P208" s="3"/>
     </row>
-    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>2313</v>
       </c>
@@ -75590,7 +75611,7 @@
       </c>
       <c r="P209" s="3"/>
     </row>
-    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>2313</v>
       </c>
@@ -75638,7 +75659,7 @@
       </c>
       <c r="P210" s="3"/>
     </row>
-    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>2313</v>
       </c>
@@ -75686,7 +75707,7 @@
       </c>
       <c r="P211" s="3"/>
     </row>
-    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>2313</v>
       </c>
@@ -75734,7 +75755,7 @@
       </c>
       <c r="P212" s="3"/>
     </row>
-    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>2313</v>
       </c>
@@ -75782,7 +75803,7 @@
       </c>
       <c r="P213" s="3"/>
     </row>
-    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>2313</v>
       </c>
@@ -75830,7 +75851,7 @@
       </c>
       <c r="P214" s="3"/>
     </row>
-    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>2313</v>
       </c>
@@ -75878,7 +75899,7 @@
       </c>
       <c r="P215" s="3"/>
     </row>
-    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>2313</v>
       </c>
@@ -75926,7 +75947,7 @@
       </c>
       <c r="P216" s="3"/>
     </row>
-    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>2313</v>
       </c>
@@ -75973,7 +75994,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>2313</v>
       </c>
@@ -76020,7 +76041,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>2313</v>
       </c>
@@ -76067,7 +76088,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>2313</v>
       </c>
@@ -76114,7 +76135,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>2313</v>
       </c>
@@ -76161,7 +76182,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>2313</v>
       </c>
@@ -76208,7 +76229,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>2313</v>
       </c>
@@ -76255,7 +76276,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>2313</v>
       </c>
@@ -76302,7 +76323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>2313</v>
       </c>
@@ -76349,7 +76370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>2313</v>
       </c>
@@ -76396,7 +76417,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>2313</v>
       </c>
@@ -76443,7 +76464,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>2313</v>
       </c>
@@ -76490,7 +76511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>2313</v>
       </c>
@@ -76537,7 +76558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>2313</v>
       </c>
@@ -76584,7 +76605,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>2313</v>
       </c>
@@ -76631,7 +76652,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>2685</v>
       </c>
@@ -76678,7 +76699,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>2654</v>
       </c>
@@ -76770,7 +76791,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>2685</v>
       </c>
@@ -76799,7 +76820,7 @@
         <v>2751</v>
       </c>
       <c r="J235" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K235" s="6" t="s">
         <v>2746</v>
@@ -76817,7 +76838,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>2685</v>
       </c>
@@ -76846,7 +76867,7 @@
         <v>2751</v>
       </c>
       <c r="J236" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K236" s="6" t="s">
         <v>2752</v>
@@ -76864,7 +76885,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>2685</v>
       </c>
@@ -76893,7 +76914,7 @@
         <v>2751</v>
       </c>
       <c r="J237" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K237" s="6" t="s">
         <v>2755</v>
@@ -76911,7 +76932,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>2685</v>
       </c>
@@ -76940,7 +76961,7 @@
         <v>2751</v>
       </c>
       <c r="J238" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K238" s="6" t="s">
         <v>2758</v>
@@ -76958,7 +76979,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>2685</v>
       </c>
@@ -76987,7 +77008,7 @@
         <v>2751</v>
       </c>
       <c r="J239" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K239" s="6" t="s">
         <v>2761</v>
@@ -77005,7 +77026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>2685</v>
       </c>
@@ -77034,7 +77055,7 @@
         <v>2751</v>
       </c>
       <c r="J240" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K240" s="6" t="s">
         <v>2764</v>
@@ -77052,7 +77073,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>2685</v>
       </c>
@@ -77081,7 +77102,7 @@
         <v>2751</v>
       </c>
       <c r="J241" t="s">
-        <v>2736</v>
+        <v>2365</v>
       </c>
       <c r="K241" s="6" t="s">
         <v>2767</v>
@@ -77099,7 +77120,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>2313</v>
       </c>
@@ -77146,7 +77167,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>2313</v>
       </c>
@@ -77193,7 +77214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>2313</v>
       </c>
@@ -77240,7 +77261,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>2313</v>
       </c>
@@ -77287,7 +77308,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>2313</v>
       </c>
@@ -77334,7 +77355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>2313</v>
       </c>
@@ -77381,7 +77402,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>2313</v>
       </c>
@@ -77428,7 +77449,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>2313</v>
       </c>
@@ -77475,7 +77496,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>2313</v>
       </c>
@@ -77522,7 +77543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>2313</v>
       </c>
@@ -77569,7 +77590,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>2313</v>
       </c>
@@ -77616,7 +77637,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>2313</v>
       </c>
@@ -77663,7 +77684,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>2313</v>
       </c>
@@ -77710,7 +77731,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>2313</v>
       </c>
@@ -77757,7 +77778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>2313</v>
       </c>
@@ -77804,7 +77825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>2313</v>
       </c>
@@ -77851,7 +77872,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="258" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A258" s="13" t="s">
         <v>2313</v>
       </c>
@@ -77898,7 +77919,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2313</v>
       </c>
@@ -77945,7 +77966,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2313</v>
       </c>
@@ -77992,7 +78013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2313</v>
       </c>
@@ -78039,7 +78060,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2313</v>
       </c>
@@ -78086,7 +78107,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2313</v>
       </c>
@@ -78133,7 +78154,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2313</v>
       </c>
@@ -78180,7 +78201,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2313</v>
       </c>
@@ -78227,7 +78248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A266" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78274,7 +78295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A267" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78321,7 +78342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A268" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78368,7 +78389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A269" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78415,7 +78436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A270" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78462,7 +78483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A271" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78509,7 +78530,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A272" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78550,7 +78571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="273" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A273" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78591,7 +78612,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="274" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A274" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78638,7 +78659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A275" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78685,7 +78706,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="276" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A276" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78732,7 +78753,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A277" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78776,7 +78797,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A278" s="11" t="s">
         <v>2313</v>
       </c>
@@ -79951,7 +79972,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2313</v>
       </c>
@@ -79964,8 +79985,8 @@
       <c r="D303" t="s">
         <v>2888</v>
       </c>
-      <c r="E303" s="22" t="s">
-        <v>2856</v>
+      <c r="E303" t="s">
+        <v>2901</v>
       </c>
       <c r="F303" t="s">
         <v>2856</v>
@@ -79985,8 +80006,8 @@
       <c r="K303" t="s">
         <v>2894</v>
       </c>
-      <c r="L303" s="22" t="s">
-        <v>2477</v>
+      <c r="L303" t="s">
+        <v>2856</v>
       </c>
       <c r="M303" t="s">
         <v>2479</v>
@@ -79998,7 +80019,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2313</v>
       </c>
@@ -80011,8 +80032,8 @@
       <c r="D304" t="s">
         <v>2889</v>
       </c>
-      <c r="E304" s="11" t="s">
-        <v>775</v>
+      <c r="E304" t="s">
+        <v>2902</v>
       </c>
       <c r="F304" t="s">
         <v>775</v>
@@ -80045,7 +80066,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2313</v>
       </c>
@@ -80058,8 +80079,8 @@
       <c r="D305" t="s">
         <v>2890</v>
       </c>
-      <c r="E305" s="22" t="s">
-        <v>2856</v>
+      <c r="E305" t="s">
+        <v>2903</v>
       </c>
       <c r="F305" t="s">
         <v>2856</v>
@@ -80079,8 +80100,8 @@
       <c r="K305" t="s">
         <v>2896</v>
       </c>
-      <c r="L305" s="22" t="s">
-        <v>2477</v>
+      <c r="L305" t="s">
+        <v>2856</v>
       </c>
       <c r="M305" t="s">
         <v>2479</v>
@@ -80092,7 +80113,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2313</v>
       </c>
@@ -80105,8 +80126,8 @@
       <c r="D306" t="s">
         <v>2891</v>
       </c>
-      <c r="E306" s="11" t="s">
-        <v>775</v>
+      <c r="E306" t="s">
+        <v>2904</v>
       </c>
       <c r="F306" t="s">
         <v>775</v>
@@ -80139,7 +80160,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2313</v>
       </c>
@@ -80152,8 +80173,8 @@
       <c r="D307" t="s">
         <v>2892</v>
       </c>
-      <c r="E307" s="22" t="s">
-        <v>2856</v>
+      <c r="E307" t="s">
+        <v>2905</v>
       </c>
       <c r="F307" t="s">
         <v>2856</v>
@@ -80173,8 +80194,8 @@
       <c r="K307" t="s">
         <v>2898</v>
       </c>
-      <c r="L307" s="22" t="s">
-        <v>2477</v>
+      <c r="L307" t="s">
+        <v>2856</v>
       </c>
       <c r="M307" t="s">
         <v>2479</v>
@@ -80186,7 +80207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="308" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2313</v>
       </c>
@@ -80199,8 +80220,8 @@
       <c r="D308" t="s">
         <v>2893</v>
       </c>
-      <c r="E308" s="22" t="s">
-        <v>2856</v>
+      <c r="E308" t="s">
+        <v>2906</v>
       </c>
       <c r="F308" t="s">
         <v>2856</v>
@@ -80220,8 +80241,8 @@
       <c r="K308" t="s">
         <v>2899</v>
       </c>
-      <c r="L308" s="22" t="s">
-        <v>2477</v>
+      <c r="L308" t="s">
+        <v>2856</v>
       </c>
       <c r="M308" t="s">
         <v>2479</v>
@@ -80234,13 +80255,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-    <filterColumn colId="12">
-      <filters>
-        <filter val="VPPyO"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}"/>
   <conditionalFormatting sqref="D278 D1:D271">
     <cfRule type="duplicateValues" dxfId="10" priority="1"/>
     <cfRule type="duplicateValues" dxfId="9" priority="11"/>

</xml_diff>

<commit_message>
Hora de actualizacion del Ppto en el header + actualiza Ppto/CECOS
- Muestra en el subtitulo del header "Ppto 2027 actualizado el DD/MM/YYYY HH:MM",
  sacado del NOMBRE del archivo (PPTO27_DD_MM_YYYY_HH_MM) via _ppto_ts() -> V2_DATA.pptoTs.
- Actualiza Ppto: PPTO27_13_07_2026_15_50.XLSX (475,871 MM) reemplaza al 15_30.
- CECOS.xlsx actualizado. Regenerados v3, BBDD y 23 dashboards + Excel por VP.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEB9DDA-6561-403F-8535-933A644FCF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DC2169-AFBB-4632-BF01-86BF7267D081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -65691,7 +65691,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:P308"/>
@@ -65764,7 +65764,7 @@
         <v>2312</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2313</v>
       </c>
@@ -65811,7 +65811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2313</v>
       </c>
@@ -65858,7 +65858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2313</v>
       </c>
@@ -65905,7 +65905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2313</v>
       </c>
@@ -65952,7 +65952,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2313</v>
       </c>
@@ -65999,7 +65999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2313</v>
       </c>
@@ -66046,7 +66046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2313</v>
       </c>
@@ -66093,7 +66093,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2313</v>
       </c>
@@ -66140,7 +66140,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2313</v>
       </c>
@@ -66187,7 +66187,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2313</v>
       </c>
@@ -66234,7 +66234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>2313</v>
       </c>
@@ -66284,7 +66284,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2313</v>
       </c>
@@ -66332,7 +66332,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>2313</v>
       </c>
@@ -66379,7 +66379,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2313</v>
       </c>
@@ -66426,7 +66426,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>2313</v>
       </c>
@@ -66473,7 +66473,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2313</v>
       </c>
@@ -66520,7 +66520,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2313</v>
       </c>
@@ -66567,7 +66567,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>2313</v>
       </c>
@@ -66614,7 +66614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2313</v>
       </c>
@@ -66661,7 +66661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>2313</v>
       </c>
@@ -66711,7 +66711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>2313</v>
       </c>
@@ -66758,7 +66758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2313</v>
       </c>
@@ -66805,7 +66805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2313</v>
       </c>
@@ -66852,7 +66852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2313</v>
       </c>
@@ -66899,7 +66899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2313</v>
       </c>
@@ -66946,7 +66946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>2313</v>
       </c>
@@ -66993,7 +66993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2313</v>
       </c>
@@ -67043,7 +67043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2313</v>
       </c>
@@ -67090,7 +67090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2313</v>
       </c>
@@ -67137,7 +67137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>2313</v>
       </c>
@@ -67184,7 +67184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2313</v>
       </c>
@@ -67234,7 +67234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2313</v>
       </c>
@@ -67281,7 +67281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>2313</v>
       </c>
@@ -67328,7 +67328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>2313</v>
       </c>
@@ -67375,7 +67375,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>2313</v>
       </c>
@@ -67422,7 +67422,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>2313</v>
       </c>
@@ -67469,7 +67469,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>2313</v>
       </c>
@@ -67516,7 +67516,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>2313</v>
       </c>
@@ -67563,7 +67563,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>2313</v>
       </c>
@@ -67610,7 +67610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>2313</v>
       </c>
@@ -67657,7 +67657,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>2313</v>
       </c>
@@ -67704,7 +67704,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>2313</v>
       </c>
@@ -67751,7 +67751,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>2313</v>
       </c>
@@ -67798,7 +67798,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>2313</v>
       </c>
@@ -67845,7 +67845,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>2313</v>
       </c>
@@ -67892,7 +67892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>2313</v>
       </c>
@@ -67939,7 +67939,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>2313</v>
       </c>
@@ -67986,7 +67986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>2313</v>
       </c>
@@ -68036,7 +68036,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>2313</v>
       </c>
@@ -68086,7 +68086,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>2313</v>
       </c>
@@ -68133,7 +68133,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>2313</v>
       </c>
@@ -68180,7 +68180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>2313</v>
       </c>
@@ -68227,7 +68227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>2313</v>
       </c>
@@ -68274,7 +68274,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>2313</v>
       </c>
@@ -68321,7 +68321,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>2313</v>
       </c>
@@ -68368,7 +68368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>2313</v>
       </c>
@@ -68415,7 +68415,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>2313</v>
       </c>
@@ -68462,7 +68462,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>2313</v>
       </c>
@@ -68509,7 +68509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>2313</v>
       </c>
@@ -68556,7 +68556,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>2313</v>
       </c>
@@ -68603,7 +68603,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>2313</v>
       </c>
@@ -68650,7 +68650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>2313</v>
       </c>
@@ -68697,7 +68697,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>2313</v>
       </c>
@@ -68744,7 +68744,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>2313</v>
       </c>
@@ -68791,7 +68791,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>2313</v>
       </c>
@@ -68838,7 +68838,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>2313</v>
       </c>
@@ -68888,7 +68888,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>2313</v>
       </c>
@@ -68935,7 +68935,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>2313</v>
       </c>
@@ -68982,7 +68982,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>2313</v>
       </c>
@@ -69029,7 +69029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>2313</v>
       </c>
@@ -69079,7 +69079,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>2313</v>
       </c>
@@ -69126,7 +69126,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>2313</v>
       </c>
@@ -69173,7 +69173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>2313</v>
       </c>
@@ -69223,7 +69223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>2313</v>
       </c>
@@ -69271,7 +69271,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>2313</v>
       </c>
@@ -69318,7 +69318,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>2313</v>
       </c>
@@ -69368,7 +69368,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>2313</v>
       </c>
@@ -69415,7 +69415,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>2313</v>
       </c>
@@ -69462,7 +69462,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>2313</v>
       </c>
@@ -69509,7 +69509,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>2313</v>
       </c>
@@ -69559,7 +69559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>2313</v>
       </c>
@@ -69609,7 +69609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>2313</v>
       </c>
@@ -69656,7 +69656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>2313</v>
       </c>
@@ -69703,7 +69703,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>2313</v>
       </c>
@@ -69750,7 +69750,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>2313</v>
       </c>
@@ -69797,7 +69797,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>2313</v>
       </c>
@@ -69844,7 +69844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>2313</v>
       </c>
@@ -69891,7 +69891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>2313</v>
       </c>
@@ -69939,7 +69939,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>2313</v>
       </c>
@@ -69987,7 +69987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>2313</v>
       </c>
@@ -70034,7 +70034,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>2313</v>
       </c>
@@ -70081,7 +70081,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>2313</v>
       </c>
@@ -70128,7 +70128,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>2313</v>
       </c>
@@ -70175,7 +70175,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>2313</v>
       </c>
@@ -70222,7 +70222,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>2313</v>
       </c>
@@ -70269,7 +70269,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>2313</v>
       </c>
@@ -70316,7 +70316,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>2313</v>
       </c>
@@ -70363,7 +70363,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>2313</v>
       </c>
@@ -70410,7 +70410,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>2313</v>
       </c>
@@ -70457,7 +70457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>2313</v>
       </c>
@@ -70504,7 +70504,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>2313</v>
       </c>
@@ -70551,7 +70551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>2313</v>
       </c>
@@ -70598,7 +70598,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>2313</v>
       </c>
@@ -70645,7 +70645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>2313</v>
       </c>
@@ -70692,7 +70692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>2313</v>
       </c>
@@ -70739,7 +70739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>2313</v>
       </c>
@@ -70789,7 +70789,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>2313</v>
       </c>
@@ -70836,7 +70836,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>2313</v>
       </c>
@@ -70883,7 +70883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>2313</v>
       </c>
@@ -70930,7 +70930,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>2313</v>
       </c>
@@ -70977,7 +70977,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>2313</v>
       </c>
@@ -71024,7 +71024,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>2313</v>
       </c>
@@ -71071,7 +71071,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>2313</v>
       </c>
@@ -71118,7 +71118,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>2313</v>
       </c>
@@ -71165,7 +71165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>2313</v>
       </c>
@@ -71212,7 +71212,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>2313</v>
       </c>
@@ -71259,7 +71259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>2313</v>
       </c>
@@ -71306,7 +71306,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>2313</v>
       </c>
@@ -71353,7 +71353,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>2313</v>
       </c>
@@ -71400,7 +71400,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>2313</v>
       </c>
@@ -71447,7 +71447,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>2313</v>
       </c>
@@ -71494,7 +71494,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>2313</v>
       </c>
@@ -71544,7 +71544,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>2313</v>
       </c>
@@ -71591,7 +71591,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>2313</v>
       </c>
@@ -71641,7 +71641,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>2313</v>
       </c>
@@ -71688,7 +71688,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>2313</v>
       </c>
@@ -71738,7 +71738,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>2313</v>
       </c>
@@ -71785,7 +71785,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71832,7 +71832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71879,7 +71879,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2313</v>
       </c>
@@ -71926,7 +71926,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>2313</v>
       </c>
@@ -71973,7 +71973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>2313</v>
       </c>
@@ -72020,7 +72020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>2313</v>
       </c>
@@ -72067,7 +72067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>2313</v>
       </c>
@@ -72114,7 +72114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>2313</v>
       </c>
@@ -72164,7 +72164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>2313</v>
       </c>
@@ -72211,7 +72211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72258,7 +72258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>2313</v>
       </c>
@@ -72305,7 +72305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>2313</v>
       </c>
@@ -72352,7 +72352,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>2313</v>
       </c>
@@ -72399,7 +72399,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>2313</v>
       </c>
@@ -72446,7 +72446,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>2313</v>
       </c>
@@ -72493,7 +72493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>2313</v>
       </c>
@@ -72540,7 +72540,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>2313</v>
       </c>
@@ -72587,7 +72587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>2313</v>
       </c>
@@ -72634,7 +72634,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72681,7 +72681,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72728,7 +72728,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>2313</v>
       </c>
@@ -72775,7 +72775,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>2313</v>
       </c>
@@ -72822,7 +72822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>2313</v>
       </c>
@@ -72869,7 +72869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>2313</v>
       </c>
@@ -72919,7 +72919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>2313</v>
       </c>
@@ -72966,7 +72966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>2313</v>
       </c>
@@ -73013,7 +73013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73060,7 +73060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>2313</v>
       </c>
@@ -73107,7 +73107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>2313</v>
       </c>
@@ -73154,7 +73154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>2313</v>
       </c>
@@ -73201,7 +73201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>2313</v>
       </c>
@@ -73248,7 +73248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>2313</v>
       </c>
@@ -73295,7 +73295,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>2313</v>
       </c>
@@ -73342,7 +73342,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>2313</v>
       </c>
@@ -73389,7 +73389,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>2313</v>
       </c>
@@ -73436,7 +73436,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>2313</v>
       </c>
@@ -73483,7 +73483,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73530,7 +73530,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73577,7 +73577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>2313</v>
       </c>
@@ -73624,7 +73624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>2313</v>
       </c>
@@ -73671,7 +73671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>2313</v>
       </c>
@@ -73718,7 +73718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>2313</v>
       </c>
@@ -73765,7 +73765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73812,7 +73812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>2313</v>
       </c>
@@ -73859,7 +73859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>2313</v>
       </c>
@@ -73909,7 +73909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>2313</v>
       </c>
@@ -73956,7 +73956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>2313</v>
       </c>
@@ -74003,7 +74003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>2313</v>
       </c>
@@ -74050,7 +74050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>2313</v>
       </c>
@@ -74097,7 +74097,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>2313</v>
       </c>
@@ -74144,7 +74144,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>2313</v>
       </c>
@@ -74191,7 +74191,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>2313</v>
       </c>
@@ -74238,7 +74238,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>2313</v>
       </c>
@@ -74285,7 +74285,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>2313</v>
       </c>
@@ -74332,7 +74332,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="183" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74379,7 +74379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74426,7 +74426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>2313</v>
       </c>
@@ -74473,7 +74473,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>2313</v>
       </c>
@@ -74520,7 +74520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>2313</v>
       </c>
@@ -74567,7 +74567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>2313</v>
       </c>
@@ -74614,7 +74614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>2313</v>
       </c>
@@ -74664,7 +74664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>2313</v>
       </c>
@@ -74711,7 +74711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74758,7 +74758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>2313</v>
       </c>
@@ -74805,7 +74805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>2313</v>
       </c>
@@ -74852,7 +74852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>2313</v>
       </c>
@@ -74899,7 +74899,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>2313</v>
       </c>
@@ -74946,7 +74946,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>2313</v>
       </c>
@@ -74993,7 +74993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>2313</v>
       </c>
@@ -75040,7 +75040,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>2313</v>
       </c>
@@ -75087,7 +75087,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>2313</v>
       </c>
@@ -75134,7 +75134,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>2313</v>
       </c>
@@ -75181,7 +75181,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>2313</v>
       </c>
@@ -75228,7 +75228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>2313</v>
       </c>
@@ -75278,7 +75278,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="203" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75325,7 +75325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="204" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75372,7 +75372,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="205" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75419,7 +75419,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>2313</v>
       </c>
@@ -75467,7 +75467,7 @@
       </c>
       <c r="P206" s="3"/>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>2313</v>
       </c>
@@ -75515,7 +75515,7 @@
       </c>
       <c r="P207" s="3"/>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>2313</v>
       </c>
@@ -75563,7 +75563,7 @@
       </c>
       <c r="P208" s="3"/>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>2313</v>
       </c>
@@ -75611,7 +75611,7 @@
       </c>
       <c r="P209" s="3"/>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>2313</v>
       </c>
@@ -75659,7 +75659,7 @@
       </c>
       <c r="P210" s="3"/>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>2313</v>
       </c>
@@ -75707,7 +75707,7 @@
       </c>
       <c r="P211" s="3"/>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>2313</v>
       </c>
@@ -75755,7 +75755,7 @@
       </c>
       <c r="P212" s="3"/>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>2313</v>
       </c>
@@ -75803,7 +75803,7 @@
       </c>
       <c r="P213" s="3"/>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>2313</v>
       </c>
@@ -75851,7 +75851,7 @@
       </c>
       <c r="P214" s="3"/>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>2313</v>
       </c>
@@ -75899,7 +75899,7 @@
       </c>
       <c r="P215" s="3"/>
     </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>2313</v>
       </c>
@@ -75947,7 +75947,7 @@
       </c>
       <c r="P216" s="3"/>
     </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>2313</v>
       </c>
@@ -75994,7 +75994,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>2313</v>
       </c>
@@ -76041,7 +76041,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>2313</v>
       </c>
@@ -76088,7 +76088,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>2313</v>
       </c>
@@ -76135,7 +76135,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>2313</v>
       </c>
@@ -76182,7 +76182,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>2313</v>
       </c>
@@ -76229,7 +76229,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>2313</v>
       </c>
@@ -76276,7 +76276,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>2313</v>
       </c>
@@ -76323,7 +76323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>2313</v>
       </c>
@@ -76370,7 +76370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>2313</v>
       </c>
@@ -76417,7 +76417,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>2313</v>
       </c>
@@ -76464,7 +76464,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>2313</v>
       </c>
@@ -76511,7 +76511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>2313</v>
       </c>
@@ -76558,7 +76558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>2313</v>
       </c>
@@ -76605,7 +76605,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>2313</v>
       </c>
@@ -76652,7 +76652,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>2685</v>
       </c>
@@ -76699,7 +76699,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>2654</v>
       </c>
@@ -76744,7 +76744,7 @@
       </c>
       <c r="P233" s="3"/>
     </row>
-    <row r="234" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>2313</v>
       </c>
@@ -77120,7 +77120,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>2313</v>
       </c>
@@ -77167,7 +77167,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>2313</v>
       </c>
@@ -77214,7 +77214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>2313</v>
       </c>
@@ -77261,7 +77261,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>2313</v>
       </c>
@@ -77308,7 +77308,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>2313</v>
       </c>
@@ -77355,7 +77355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>2313</v>
       </c>
@@ -77402,7 +77402,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>2313</v>
       </c>
@@ -77449,7 +77449,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>2313</v>
       </c>
@@ -77496,7 +77496,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>2313</v>
       </c>
@@ -77543,7 +77543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>2313</v>
       </c>
@@ -77590,7 +77590,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>2313</v>
       </c>
@@ -77637,7 +77637,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>2313</v>
       </c>
@@ -77684,7 +77684,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>2313</v>
       </c>
@@ -77731,7 +77731,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>2313</v>
       </c>
@@ -77778,7 +77778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>2313</v>
       </c>
@@ -77825,7 +77825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="257" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>2313</v>
       </c>
@@ -77872,7 +77872,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="258" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" s="13" t="s">
         <v>2313</v>
       </c>
@@ -77919,7 +77919,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2313</v>
       </c>
@@ -77966,7 +77966,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="260" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2313</v>
       </c>
@@ -78013,7 +78013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2313</v>
       </c>
@@ -78060,7 +78060,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2313</v>
       </c>
@@ -78107,7 +78107,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2313</v>
       </c>
@@ -78154,7 +78154,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2313</v>
       </c>
@@ -78201,7 +78201,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2313</v>
       </c>
@@ -78248,7 +78248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78295,7 +78295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78342,7 +78342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78389,7 +78389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78436,7 +78436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78483,7 +78483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78552,8 +78552,8 @@
       <c r="G272" s="11" t="s">
         <v>2749</v>
       </c>
-      <c r="J272" s="11" t="s">
-        <v>2736</v>
+      <c r="J272" t="s">
+        <v>2365</v>
       </c>
       <c r="K272" s="11" t="s">
         <v>2824</v>
@@ -78593,8 +78593,8 @@
       <c r="G273" s="11" t="s">
         <v>2749</v>
       </c>
-      <c r="J273" s="11" t="s">
-        <v>2736</v>
+      <c r="J273" t="s">
+        <v>2365</v>
       </c>
       <c r="K273" s="11" t="s">
         <v>2827</v>
@@ -78640,8 +78640,8 @@
       <c r="I274" s="11" t="s">
         <v>2751</v>
       </c>
-      <c r="J274" s="11" t="s">
-        <v>2736</v>
+      <c r="J274" t="s">
+        <v>2365</v>
       </c>
       <c r="K274" s="11" t="s">
         <v>2832</v>
@@ -78659,7 +78659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78706,7 +78706,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="276" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78753,7 +78753,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78797,7 +78797,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78844,7 +78844,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>2313</v>
       </c>
@@ -78891,7 +78891,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>2313</v>
       </c>
@@ -78938,7 +78938,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>2313</v>
       </c>
@@ -78985,7 +78985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>2313</v>
       </c>
@@ -79032,7 +79032,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>2313</v>
       </c>
@@ -79079,7 +79079,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>2313</v>
       </c>
@@ -79126,7 +79126,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>2313</v>
       </c>
@@ -79173,7 +79173,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>2313</v>
       </c>
@@ -79220,7 +79220,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>2313</v>
       </c>
@@ -79267,7 +79267,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>2313</v>
       </c>
@@ -79314,7 +79314,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>2313</v>
       </c>
@@ -79361,7 +79361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>2313</v>
       </c>
@@ -79408,7 +79408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>2313</v>
       </c>
@@ -79455,7 +79455,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>2313</v>
       </c>
@@ -79502,7 +79502,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>2313</v>
       </c>
@@ -79549,7 +79549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>2313</v>
       </c>
@@ -79596,7 +79596,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="295" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>2313</v>
       </c>
@@ -79643,7 +79643,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>2313</v>
       </c>
@@ -79690,7 +79690,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>2313</v>
       </c>
@@ -79737,7 +79737,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>2313</v>
       </c>
@@ -79784,7 +79784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>2313</v>
       </c>
@@ -79831,7 +79831,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>2313</v>
       </c>
@@ -79878,7 +79878,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>2313</v>
       </c>
@@ -79925,7 +79925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="302" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>2313</v>
       </c>
@@ -79972,7 +79972,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2313</v>
       </c>
@@ -80019,7 +80019,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2313</v>
       </c>
@@ -80066,7 +80066,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2313</v>
       </c>
@@ -80113,7 +80113,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="306" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2313</v>
       </c>
@@ -80160,7 +80160,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2313</v>
       </c>
@@ -80207,7 +80207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="308" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2313</v>
       </c>
@@ -80255,7 +80255,22 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}"/>
+  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="1000AP0419"/>
+        <filter val="1000AP0501"/>
+        <filter val="1000AP0502"/>
+        <filter val="1000AP0503"/>
+        <filter val="1000AP0508"/>
+        <filter val="1000AP0509"/>
+        <filter val="1000AP0513"/>
+        <filter val="1000AP0514"/>
+        <filter val="1000AP0517"/>
+        <filter val="1000AP0518"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="D278 D1:D271">
     <cfRule type="duplicateValues" dxfId="10" priority="1"/>
     <cfRule type="duplicateValues" dxfId="9" priority="11"/>
@@ -80296,15 +80311,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="70b3a8a4-10f1-4453-b557-059c8aa2e01d" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -80569,21 +80581,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="70b3a8a4-10f1-4453-b557-059c8aa2e01d" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
-    <ds:schemaRef ds:uri="70b3a8a4-10f1-4453-b557-059c8aa2e01d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -80608,9 +80620,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
+    <ds:schemaRef ds:uri="70b3a8a4-10f1-4453-b557-059c8aa2e01d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualiza nombres en CECOS
- CECOS.xlsx: cambios de nombres (VP / Gerencia / Desc. CECO).
- Regenerados v3, BBDD (dim_cecos) y los 23 dashboards + subvista TICA + Excels por VP.
  Solo cambio dim_cecos entre los parquet (los hechos no dependen de los nombres).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DC2169-AFBB-4632-BF01-86BF7267D081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAC9C666-2F2B-4C52-9714-C09FA0473245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19682" uniqueCount="2907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19682" uniqueCount="2912">
   <si>
     <t>Clasificación 1</t>
   </si>
@@ -8766,6 +8766,21 @@
   </si>
   <si>
     <t>Compliance CMZ</t>
+  </si>
+  <si>
+    <t>Protección industrial</t>
+  </si>
+  <si>
+    <t>AAPP Norte</t>
+  </si>
+  <si>
+    <t>RRII</t>
+  </si>
+  <si>
+    <t>Distribuibles Corporativos</t>
+  </si>
+  <si>
+    <t>FMLP</t>
   </si>
 </sst>
 </file>
@@ -8775,7 +8790,7 @@
   <numFmts count="1">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8929,6 +8944,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="40">
@@ -9154,7 +9182,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -9284,8 +9312,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="63">
+  <cellStyleXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -9349,8 +9386,10 @@
     <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -9423,8 +9462,11 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="63" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="63">
+  <cellStyles count="65">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis1 2" xfId="45" xr:uid="{3084E8CE-3FDA-47A2-8840-2F1A6BE152B9}"/>
     <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
@@ -9479,8 +9521,10 @@
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="42" xr:uid="{3C0EEC1D-5B9D-46C9-A4FC-5E40667FF5C3}"/>
+    <cellStyle name="Normal 3" xfId="63" xr:uid="{EB80B8F5-C6F3-4772-A276-6B14C8AE50CD}"/>
     <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Notas 2" xfId="44" xr:uid="{C5BDD28A-B719-49C0-A8E5-6C235E43AA8A}"/>
+    <cellStyle name="Porcentaje 2" xfId="64" xr:uid="{18CFB098-6C82-45CE-A819-FA401A4C633C}"/>
     <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
@@ -10018,6 +10062,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="5">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{E857A7B1-2B0E-4DDF-A7BD-4A9FBEBDF655}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;091344bf-97b7-40e7-95e4-a4f547f6faf9&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC70E907-DA9C-4B4F-99E4-5967E1F483B7}">
   <sheetPr codeName="Hoja1"/>
@@ -68215,7 +68281,7 @@
         <v>2453</v>
       </c>
       <c r="L53" t="s">
-        <v>2452</v>
+        <v>2617</v>
       </c>
       <c r="M53" t="s">
         <v>2454</v>
@@ -68262,7 +68328,7 @@
         <v>2453</v>
       </c>
       <c r="L54" t="s">
-        <v>2452</v>
+        <v>2619</v>
       </c>
       <c r="M54" t="s">
         <v>2454</v>
@@ -68356,7 +68422,7 @@
         <v>2453</v>
       </c>
       <c r="L56" t="s">
-        <v>2452</v>
+        <v>2907</v>
       </c>
       <c r="M56" t="s">
         <v>2454</v>
@@ -70189,7 +70255,7 @@
         <v>2575</v>
       </c>
       <c r="E95" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F95" t="s">
         <v>2577</v>
@@ -70210,7 +70276,7 @@
         <v>2581</v>
       </c>
       <c r="L95" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M95" t="s">
         <v>2454</v>
@@ -70236,7 +70302,7 @@
         <v>2584</v>
       </c>
       <c r="E96" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F96" t="s">
         <v>2577</v>
@@ -70257,7 +70323,7 @@
         <v>2581</v>
       </c>
       <c r="L96" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M96" t="s">
         <v>2454</v>
@@ -70282,7 +70348,7 @@
       <c r="D97" t="s">
         <v>2585</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E97" s="32" t="s">
         <v>2586</v>
       </c>
       <c r="F97" t="s">
@@ -70304,7 +70370,7 @@
         <v>2581</v>
       </c>
       <c r="L97" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M97" t="s">
         <v>2454</v>
@@ -70330,7 +70396,7 @@
         <v>2587</v>
       </c>
       <c r="E98" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F98" t="s">
         <v>2577</v>
@@ -70351,7 +70417,7 @@
         <v>2588</v>
       </c>
       <c r="L98" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M98" t="s">
         <v>2454</v>
@@ -70377,7 +70443,7 @@
         <v>2589</v>
       </c>
       <c r="E99" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F99" t="s">
         <v>2590</v>
@@ -70398,7 +70464,7 @@
         <v>2588</v>
       </c>
       <c r="L99" t="s">
-        <v>2590</v>
+        <v>2609</v>
       </c>
       <c r="M99" t="s">
         <v>2454</v>
@@ -70424,7 +70490,7 @@
         <v>2591</v>
       </c>
       <c r="E100" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F100" t="s">
         <v>2592</v>
@@ -70445,7 +70511,7 @@
         <v>2588</v>
       </c>
       <c r="L100" t="s">
-        <v>2592</v>
+        <v>2609</v>
       </c>
       <c r="M100" t="s">
         <v>2454</v>
@@ -70471,7 +70537,7 @@
         <v>2593</v>
       </c>
       <c r="E101" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F101" t="s">
         <v>2577</v>
@@ -70492,7 +70558,7 @@
         <v>2594</v>
       </c>
       <c r="L101" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M101" t="s">
         <v>2454</v>
@@ -70518,7 +70584,7 @@
         <v>2595</v>
       </c>
       <c r="E102" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F102" t="s">
         <v>2577</v>
@@ -70539,7 +70605,7 @@
         <v>2594</v>
       </c>
       <c r="L102" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M102" t="s">
         <v>2454</v>
@@ -70586,7 +70652,7 @@
         <v>2594</v>
       </c>
       <c r="L103" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M103" t="s">
         <v>2454</v>
@@ -70611,8 +70677,8 @@
       <c r="D104" t="s">
         <v>2598</v>
       </c>
-      <c r="E104" t="s">
-        <v>2599</v>
+      <c r="E104" s="32" t="s">
+        <v>2911</v>
       </c>
       <c r="F104" t="s">
         <v>2577</v>
@@ -70633,7 +70699,7 @@
         <v>2600</v>
       </c>
       <c r="L104" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M104" t="s">
         <v>2454</v>
@@ -70658,7 +70724,7 @@
       <c r="D105" t="s">
         <v>2601</v>
       </c>
-      <c r="E105" t="s">
+      <c r="E105" s="32" t="s">
         <v>2586</v>
       </c>
       <c r="F105" t="s">
@@ -70680,7 +70746,7 @@
         <v>2600</v>
       </c>
       <c r="L105" t="s">
-        <v>2602</v>
+        <v>2609</v>
       </c>
       <c r="M105" t="s">
         <v>2454</v>
@@ -70727,7 +70793,7 @@
         <v>2600</v>
       </c>
       <c r="L106" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M106" t="s">
         <v>2454</v>
@@ -70752,8 +70818,8 @@
       <c r="D107" t="s">
         <v>2604</v>
       </c>
-      <c r="E107" t="s">
-        <v>2605</v>
+      <c r="E107" s="32" t="s">
+        <v>361</v>
       </c>
       <c r="F107" t="s">
         <v>2606</v>
@@ -70774,7 +70840,7 @@
         <v>2600</v>
       </c>
       <c r="L107" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="M107" t="s">
         <v>2454</v>
@@ -70803,7 +70869,7 @@
         <v>2607</v>
       </c>
       <c r="E108" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F108" t="s">
         <v>2577</v>
@@ -70824,7 +70890,7 @@
         <v>2600</v>
       </c>
       <c r="L108" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M108" t="s">
         <v>2454</v>
@@ -70849,7 +70915,7 @@
       <c r="D109" t="s">
         <v>2608</v>
       </c>
-      <c r="E109" t="s">
+      <c r="E109" s="32" t="s">
         <v>2586</v>
       </c>
       <c r="F109" t="s">
@@ -70897,7 +70963,7 @@
         <v>2610</v>
       </c>
       <c r="E110" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="F110" t="s">
         <v>2577</v>
@@ -70918,7 +70984,7 @@
         <v>2600</v>
       </c>
       <c r="L110" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M110" t="s">
         <v>2454</v>
@@ -70944,7 +71010,7 @@
         <v>2611</v>
       </c>
       <c r="E111" t="s">
-        <v>2612</v>
+        <v>2577</v>
       </c>
       <c r="F111" t="s">
         <v>2456</v>
@@ -70965,7 +71031,7 @@
         <v>2613</v>
       </c>
       <c r="L111" t="s">
-        <v>2615</v>
+        <v>2908</v>
       </c>
       <c r="M111" t="s">
         <v>2454</v>
@@ -70990,8 +71056,8 @@
       <c r="D112" t="s">
         <v>2616</v>
       </c>
-      <c r="E112" t="s">
-        <v>2617</v>
+      <c r="E112" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F112" t="s">
         <v>2456</v>
@@ -71012,7 +71078,7 @@
         <v>2613</v>
       </c>
       <c r="L112" t="s">
-        <v>2617</v>
+        <v>2908</v>
       </c>
       <c r="M112" t="s">
         <v>2454</v>
@@ -71037,8 +71103,8 @@
       <c r="D113" t="s">
         <v>2618</v>
       </c>
-      <c r="E113" t="s">
-        <v>2619</v>
+      <c r="E113" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F113" t="s">
         <v>2458</v>
@@ -71059,7 +71125,7 @@
         <v>2613</v>
       </c>
       <c r="L113" t="s">
-        <v>2620</v>
+        <v>2908</v>
       </c>
       <c r="M113" t="s">
         <v>2454</v>
@@ -71084,8 +71150,8 @@
       <c r="D114" t="s">
         <v>2621</v>
       </c>
-      <c r="E114" t="s">
-        <v>2622</v>
+      <c r="E114" s="32" t="s">
+        <v>2909</v>
       </c>
       <c r="F114" t="s">
         <v>2456</v>
@@ -71106,7 +71172,7 @@
         <v>2613</v>
       </c>
       <c r="L114" t="s">
-        <v>2622</v>
+        <v>2908</v>
       </c>
       <c r="M114" t="s">
         <v>2454</v>
@@ -71132,7 +71198,7 @@
         <v>2623</v>
       </c>
       <c r="E115" t="s">
-        <v>2612</v>
+        <v>2577</v>
       </c>
       <c r="F115" t="s">
         <v>2456</v>
@@ -71153,7 +71219,7 @@
         <v>2624</v>
       </c>
       <c r="L115" t="s">
-        <v>2626</v>
+        <v>2908</v>
       </c>
       <c r="M115" t="s">
         <v>2454</v>
@@ -71178,8 +71244,8 @@
       <c r="D116" t="s">
         <v>2627</v>
       </c>
-      <c r="E116" t="s">
-        <v>2617</v>
+      <c r="E116" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F116" t="s">
         <v>2456</v>
@@ -71200,7 +71266,7 @@
         <v>2624</v>
       </c>
       <c r="L116" t="s">
-        <v>2617</v>
+        <v>2908</v>
       </c>
       <c r="M116" t="s">
         <v>2454</v>
@@ -71225,8 +71291,8 @@
       <c r="D117" t="s">
         <v>2628</v>
       </c>
-      <c r="E117" t="s">
-        <v>2619</v>
+      <c r="E117" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F117" t="s">
         <v>2458</v>
@@ -71247,7 +71313,7 @@
         <v>2624</v>
       </c>
       <c r="L117" t="s">
-        <v>2629</v>
+        <v>2908</v>
       </c>
       <c r="M117" t="s">
         <v>2454</v>
@@ -71272,8 +71338,8 @@
       <c r="D118" t="s">
         <v>2630</v>
       </c>
-      <c r="E118" t="s">
-        <v>2622</v>
+      <c r="E118" s="32" t="s">
+        <v>2909</v>
       </c>
       <c r="F118" t="s">
         <v>2456</v>
@@ -71294,7 +71360,7 @@
         <v>2624</v>
       </c>
       <c r="L118" t="s">
-        <v>2622</v>
+        <v>2908</v>
       </c>
       <c r="M118" t="s">
         <v>2454</v>
@@ -71341,7 +71407,7 @@
         <v>2635</v>
       </c>
       <c r="L119" t="s">
-        <v>2632</v>
+        <v>2908</v>
       </c>
       <c r="M119" t="s">
         <v>2454</v>
@@ -71366,8 +71432,8 @@
       <c r="D120" t="s">
         <v>2636</v>
       </c>
-      <c r="E120" t="s">
-        <v>2617</v>
+      <c r="E120" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F120" t="s">
         <v>2456</v>
@@ -71388,7 +71454,7 @@
         <v>2635</v>
       </c>
       <c r="L120" t="s">
-        <v>2617</v>
+        <v>2908</v>
       </c>
       <c r="M120" t="s">
         <v>2454</v>
@@ -71413,8 +71479,8 @@
       <c r="D121" t="s">
         <v>2637</v>
       </c>
-      <c r="E121" t="s">
-        <v>2619</v>
+      <c r="E121" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F121" t="s">
         <v>2458</v>
@@ -71435,7 +71501,7 @@
         <v>2635</v>
       </c>
       <c r="L121" t="s">
-        <v>2620</v>
+        <v>2908</v>
       </c>
       <c r="M121" t="s">
         <v>2454</v>
@@ -71460,8 +71526,8 @@
       <c r="D122" t="s">
         <v>2638</v>
       </c>
-      <c r="E122" t="s">
-        <v>2622</v>
+      <c r="E122" s="32" t="s">
+        <v>2909</v>
       </c>
       <c r="F122" t="s">
         <v>2456</v>
@@ -71482,7 +71548,7 @@
         <v>2635</v>
       </c>
       <c r="L122" t="s">
-        <v>2622</v>
+        <v>2908</v>
       </c>
       <c r="M122" t="s">
         <v>2454</v>
@@ -72318,8 +72384,8 @@
       <c r="D140" t="s">
         <v>720</v>
       </c>
-      <c r="E140" t="s">
-        <v>721</v>
+      <c r="E140" s="32" t="s">
+        <v>361</v>
       </c>
       <c r="F140" t="s">
         <v>2577</v>
@@ -72340,7 +72406,7 @@
         <v>720</v>
       </c>
       <c r="L140" t="s">
-        <v>2582</v>
+        <v>2609</v>
       </c>
       <c r="M140" t="s">
         <v>2454</v>
@@ -72365,7 +72431,7 @@
       <c r="D141" t="s">
         <v>722</v>
       </c>
-      <c r="E141" t="s">
+      <c r="E141" s="32" t="s">
         <v>361</v>
       </c>
       <c r="F141" t="s">
@@ -73167,8 +73233,8 @@
       <c r="D158" t="s">
         <v>1794</v>
       </c>
-      <c r="E158" t="s">
-        <v>1795</v>
+      <c r="E158" s="32" t="s">
+        <v>2586</v>
       </c>
       <c r="F158" t="s">
         <v>2458</v>
@@ -73189,7 +73255,7 @@
         <v>1794</v>
       </c>
       <c r="L158" t="s">
-        <v>2670</v>
+        <v>2908</v>
       </c>
       <c r="M158" t="s">
         <v>2454</v>
@@ -73261,8 +73327,8 @@
       <c r="D160" t="s">
         <v>1797</v>
       </c>
-      <c r="E160" t="s">
-        <v>2671</v>
+      <c r="E160" s="32" t="s">
+        <v>361</v>
       </c>
       <c r="F160" t="s">
         <v>1798</v>
@@ -73283,7 +73349,7 @@
         <v>1797</v>
       </c>
       <c r="L160" t="s">
-        <v>1798</v>
+        <v>2908</v>
       </c>
       <c r="M160" t="s">
         <v>2454</v>
@@ -74063,8 +74129,8 @@
       <c r="D177" t="s">
         <v>2063</v>
       </c>
-      <c r="E177" t="s">
-        <v>2064</v>
+      <c r="E177" s="32" t="s">
+        <v>2586</v>
       </c>
       <c r="F177" t="s">
         <v>2673</v>
@@ -74085,7 +74151,7 @@
         <v>2063</v>
       </c>
       <c r="L177" t="s">
-        <v>2673</v>
+        <v>2908</v>
       </c>
       <c r="M177" t="s">
         <v>2454</v>
@@ -74251,8 +74317,8 @@
       <c r="D181" t="s">
         <v>2081</v>
       </c>
-      <c r="E181" t="s">
-        <v>2671</v>
+      <c r="E181" s="32" t="s">
+        <v>361</v>
       </c>
       <c r="F181" t="s">
         <v>1798</v>
@@ -74273,7 +74339,7 @@
         <v>2081</v>
       </c>
       <c r="L181" t="s">
-        <v>1798</v>
+        <v>2908</v>
       </c>
       <c r="M181" t="s">
         <v>2454</v>
@@ -74959,8 +75025,8 @@
       <c r="D196" t="s">
         <v>2282</v>
       </c>
-      <c r="E196" t="s">
-        <v>2675</v>
+      <c r="E196" s="32" t="s">
+        <v>2586</v>
       </c>
       <c r="F196" t="s">
         <v>2632</v>
@@ -74981,7 +75047,7 @@
         <v>2282</v>
       </c>
       <c r="L196" t="s">
-        <v>2632</v>
+        <v>2908</v>
       </c>
       <c r="M196" t="s">
         <v>2454</v>
@@ -75053,8 +75119,8 @@
       <c r="D198" t="s">
         <v>2286</v>
       </c>
-      <c r="E198" t="s">
-        <v>2671</v>
+      <c r="E198" s="32" t="s">
+        <v>361</v>
       </c>
       <c r="F198" t="s">
         <v>1798</v>
@@ -75075,7 +75141,7 @@
         <v>2286</v>
       </c>
       <c r="L198" t="s">
-        <v>1798</v>
+        <v>2908</v>
       </c>
       <c r="M198" t="s">
         <v>2454</v>
@@ -76820,7 +76886,7 @@
         <v>2751</v>
       </c>
       <c r="J235" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K235" s="6" t="s">
         <v>2746</v>
@@ -76867,7 +76933,7 @@
         <v>2751</v>
       </c>
       <c r="J236" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K236" s="6" t="s">
         <v>2752</v>
@@ -76914,7 +76980,7 @@
         <v>2751</v>
       </c>
       <c r="J237" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K237" s="6" t="s">
         <v>2755</v>
@@ -76961,7 +77027,7 @@
         <v>2751</v>
       </c>
       <c r="J238" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K238" s="6" t="s">
         <v>2758</v>
@@ -77008,7 +77074,7 @@
         <v>2751</v>
       </c>
       <c r="J239" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K239" s="6" t="s">
         <v>2761</v>
@@ -77055,7 +77121,7 @@
         <v>2751</v>
       </c>
       <c r="J240" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K240" s="6" t="s">
         <v>2764</v>
@@ -77102,7 +77168,7 @@
         <v>2751</v>
       </c>
       <c r="J241" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K241" s="6" t="s">
         <v>2767</v>
@@ -77368,8 +77434,8 @@
       <c r="D247" s="6" t="s">
         <v>2789</v>
       </c>
-      <c r="E247" t="s">
-        <v>2619</v>
+      <c r="E247" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F247" t="s">
         <v>2619</v>
@@ -77390,7 +77456,7 @@
         <v>2600</v>
       </c>
       <c r="L247" t="s">
-        <v>2773</v>
+        <v>2609</v>
       </c>
       <c r="M247" t="s">
         <v>2454</v>
@@ -77415,8 +77481,8 @@
       <c r="D248" s="6" t="s">
         <v>2790</v>
       </c>
-      <c r="E248" t="s">
-        <v>2617</v>
+      <c r="E248" s="32" t="s">
+        <v>2910</v>
       </c>
       <c r="F248" t="s">
         <v>2617</v>
@@ -77437,7 +77503,7 @@
         <v>2600</v>
       </c>
       <c r="L248" t="s">
-        <v>2773</v>
+        <v>2609</v>
       </c>
       <c r="M248" t="s">
         <v>2454</v>
@@ -78553,7 +78619,7 @@
         <v>2749</v>
       </c>
       <c r="J272" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K272" s="11" t="s">
         <v>2824</v>
@@ -78594,7 +78660,7 @@
         <v>2749</v>
       </c>
       <c r="J273" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K273" s="11" t="s">
         <v>2827</v>
@@ -78641,7 +78707,7 @@
         <v>2751</v>
       </c>
       <c r="J274" t="s">
-        <v>2365</v>
+        <v>2736</v>
       </c>
       <c r="K274" s="11" t="s">
         <v>2832</v>
@@ -80256,9 +80322,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-    <filterColumn colId="10">
+    <filterColumn colId="3">
       <filters>
-        <filter val="1000AP0419"/>
         <filter val="1000AP0501"/>
         <filter val="1000AP0502"/>
         <filter val="1000AP0503"/>
@@ -80268,6 +80333,7 @@
         <filter val="1000AP0514"/>
         <filter val="1000AP0517"/>
         <filter val="1000AP0518"/>
+        <filter val="1000AP0519"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Aplica rename de CECOS (VPAC) + regenera solo VP Asuntos Corporativos
- CECOS.xlsx: gerencia del CECO 1000AC4501 -> "VPAC" (VP Asuntos Corporativos).
- Reconstruye v3 + BBDD (dim_cecos) y regenera SOLO el dashboard de VP Asuntos Corporativos
  (los demas por-VP no cambian: su data no se toco).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAC9C666-2F2B-4C52-9714-C09FA0473245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A838F1CE-BAC7-4A9B-8348-807B46C40442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -68199,7 +68199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>2313</v>
       </c>
@@ -68234,7 +68234,7 @@
         <v>2453</v>
       </c>
       <c r="L52" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="M52" t="s">
         <v>2454</v>
@@ -68246,7 +68246,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>2313</v>
       </c>
@@ -68293,7 +68293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>2313</v>
       </c>
@@ -68387,7 +68387,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>2313</v>
       </c>
@@ -68481,7 +68481,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>2313</v>
       </c>
@@ -68528,7 +68528,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>2313</v>
       </c>
@@ -68954,7 +68954,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>2313</v>
       </c>
@@ -75294,7 +75294,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>2313</v>
       </c>
@@ -76342,7 +76342,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>2313</v>
       </c>
@@ -76857,7 +76857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>2685</v>
       </c>
@@ -76904,7 +76904,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>2685</v>
       </c>
@@ -76951,7 +76951,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>2685</v>
       </c>
@@ -76998,7 +76998,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>2685</v>
       </c>
@@ -77045,7 +77045,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>2685</v>
       </c>
@@ -77092,7 +77092,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>2685</v>
       </c>
@@ -77139,7 +77139,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>2685</v>
       </c>
@@ -77186,7 +77186,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>2313</v>
       </c>
@@ -77515,7 +77515,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>2313</v>
       </c>
@@ -77750,7 +77750,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>2313</v>
       </c>
@@ -77985,7 +77985,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2313</v>
       </c>
@@ -78549,7 +78549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A271" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78596,7 +78596,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78637,7 +78637,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="273" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78678,7 +78678,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="274" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="11" t="s">
         <v>2685</v>
       </c>
@@ -80324,16 +80324,25 @@
   <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
     <filterColumn colId="3">
       <filters>
-        <filter val="1000AP0501"/>
-        <filter val="1000AP0502"/>
-        <filter val="1000AP0503"/>
-        <filter val="1000AP0508"/>
-        <filter val="1000AP0509"/>
-        <filter val="1000AP0513"/>
-        <filter val="1000AP0514"/>
-        <filter val="1000AP0517"/>
-        <filter val="1000AP0518"/>
-        <filter val="1000AP0519"/>
+        <filter val="1000AC0520"/>
+        <filter val="1000AC4501"/>
+        <filter val="1000AC4502"/>
+        <filter val="1000AC4503"/>
+        <filter val="1000AC4505"/>
+        <filter val="1000AC4507"/>
+        <filter val="1000AC4508"/>
+        <filter val="1001AD0506"/>
+        <filter val="1001AD4527"/>
+        <filter val="1001AD4540"/>
+        <filter val="1002AD0507"/>
+        <filter val="1003AD0507"/>
+        <filter val="1003AD4500"/>
+        <filter val="1005AD0508"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="VP Asuntos Corporativos"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -80377,12 +80386,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="70b3a8a4-10f1-4453-b557-059c8aa2e01d" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -80647,21 +80659,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="70b3a8a4-10f1-4453-b557-059c8aa2e01d" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
+    <ds:schemaRef ds:uri="70b3a8a4-10f1-4453-b557-059c8aa2e01d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -80686,12 +80698,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
-    <ds:schemaRef ds:uri="70b3a8a4-10f1-4453-b557-059c8aa2e01d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Vista combinada para VP Desarrollo de Negocios + CECOS (308)
- dividir_por_vp: VISTAS_COMBINADAS. El dashboard de "VP Desarrollo de Negocios e Innovacion"
  ahora cruza 6 alcances: esa VP + VP Planif. y Serv. Tec. + VP Exploraciones y Rec. Mineros +
  Exploraciones + (sin VP) + de VP Finanzas solo TICA + TICA Corporativo. Reemplaza el dashboard
  estandar de esa VP (90 CECOs, 9430 regs).
- CECOS.xlsx: +1 CECO (1000AC7017 en VP Desarrollo; 307 -> 308). Regenerado v3 + BBDD (dim_cecos).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A838F1CE-BAC7-4A9B-8348-807B46C40442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEDAA5F-CFEE-4C6A-939F-0A9461A9379C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19682" uniqueCount="2912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19696" uniqueCount="2913">
   <si>
     <t>Clasificación 1</t>
   </si>
@@ -8781,14 +8781,18 @@
   </si>
   <si>
     <t>FMLP</t>
+  </si>
+  <si>
+    <t>1000AC7017</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="23" x14ac:knownFonts="1">
     <font>
@@ -9322,7 +9326,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="65">
+  <cellStyleXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -9388,8 +9392,9 @@
     <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -9465,8 +9470,17 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="63" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="65">
+  <cellStyles count="66">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis1 2" xfId="45" xr:uid="{3084E8CE-3FDA-47A2-8840-2F1A6BE152B9}"/>
     <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
@@ -9518,6 +9532,7 @@
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Millares [0] 2" xfId="43" xr:uid="{62963445-5FBA-42E7-9551-AD124DBB842C}"/>
+    <cellStyle name="Millares [0] 2 2" xfId="65" xr:uid="{9772BCB5-A509-4620-B80A-42A3B9FC6FD1}"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="42" xr:uid="{3C0EEC1D-5B9D-46C9-A4FC-5E40667FF5C3}"/>
@@ -65757,10 +65772,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:P308"/>
+  <dimension ref="A1:P309"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.44140625" customWidth="1"/>
@@ -65830,7 +65845,7 @@
         <v>2312</v>
       </c>
     </row>
-    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2313</v>
       </c>
@@ -65877,7 +65892,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2313</v>
       </c>
@@ -65924,7 +65939,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2313</v>
       </c>
@@ -65971,7 +65986,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2313</v>
       </c>
@@ -66018,7 +66033,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2313</v>
       </c>
@@ -66065,7 +66080,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2313</v>
       </c>
@@ -66112,7 +66127,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2313</v>
       </c>
@@ -66159,7 +66174,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2313</v>
       </c>
@@ -66206,7 +66221,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2313</v>
       </c>
@@ -66253,7 +66268,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2313</v>
       </c>
@@ -66300,7 +66315,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>2313</v>
       </c>
@@ -66350,7 +66365,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2313</v>
       </c>
@@ -66398,7 +66413,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>2313</v>
       </c>
@@ -66445,7 +66460,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2313</v>
       </c>
@@ -66492,7 +66507,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>2313</v>
       </c>
@@ -66539,7 +66554,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2313</v>
       </c>
@@ -66586,7 +66601,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2313</v>
       </c>
@@ -66633,7 +66648,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>2313</v>
       </c>
@@ -66680,7 +66695,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2313</v>
       </c>
@@ -66727,7 +66742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>2313</v>
       </c>
@@ -66777,7 +66792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>2313</v>
       </c>
@@ -66824,7 +66839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2313</v>
       </c>
@@ -66871,7 +66886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2313</v>
       </c>
@@ -66918,7 +66933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2313</v>
       </c>
@@ -66965,7 +66980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2313</v>
       </c>
@@ -67012,7 +67027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>2313</v>
       </c>
@@ -67059,7 +67074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2313</v>
       </c>
@@ -67109,7 +67124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2313</v>
       </c>
@@ -67156,7 +67171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2313</v>
       </c>
@@ -67203,7 +67218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>2313</v>
       </c>
@@ -67250,7 +67265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2313</v>
       </c>
@@ -67300,7 +67315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2313</v>
       </c>
@@ -67347,7 +67362,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>2313</v>
       </c>
@@ -67394,7 +67409,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>2313</v>
       </c>
@@ -67441,7 +67456,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>2313</v>
       </c>
@@ -67488,7 +67503,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>2313</v>
       </c>
@@ -67535,7 +67550,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>2313</v>
       </c>
@@ -67582,7 +67597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>2313</v>
       </c>
@@ -67629,7 +67644,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>2313</v>
       </c>
@@ -67676,7 +67691,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>2313</v>
       </c>
@@ -67723,7 +67738,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>2313</v>
       </c>
@@ -67770,7 +67785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>2313</v>
       </c>
@@ -67817,7 +67832,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>2313</v>
       </c>
@@ -67864,7 +67879,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>2313</v>
       </c>
@@ -67911,7 +67926,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>2313</v>
       </c>
@@ -67958,7 +67973,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>2313</v>
       </c>
@@ -68005,7 +68020,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>2313</v>
       </c>
@@ -68052,7 +68067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>2313</v>
       </c>
@@ -68102,7 +68117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>2313</v>
       </c>
@@ -68152,7 +68167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>2313</v>
       </c>
@@ -68340,7 +68355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>2313</v>
       </c>
@@ -68434,7 +68449,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>2313</v>
       </c>
@@ -68575,7 +68590,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>2313</v>
       </c>
@@ -68622,7 +68637,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>2313</v>
       </c>
@@ -68669,7 +68684,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>2313</v>
       </c>
@@ -68716,7 +68731,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>2313</v>
       </c>
@@ -68763,7 +68778,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>2313</v>
       </c>
@@ -68810,7 +68825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>2313</v>
       </c>
@@ -68857,7 +68872,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>2313</v>
       </c>
@@ -68904,7 +68919,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>2313</v>
       </c>
@@ -69001,7 +69016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>2313</v>
       </c>
@@ -69048,7 +69063,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>2313</v>
       </c>
@@ -69095,7 +69110,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>2313</v>
       </c>
@@ -69145,7 +69160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>2313</v>
       </c>
@@ -69192,7 +69207,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>2313</v>
       </c>
@@ -69239,7 +69254,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>2313</v>
       </c>
@@ -69289,7 +69304,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>2313</v>
       </c>
@@ -69337,7 +69352,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>2313</v>
       </c>
@@ -69384,7 +69399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>2313</v>
       </c>
@@ -69434,7 +69449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>2313</v>
       </c>
@@ -69481,7 +69496,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>2313</v>
       </c>
@@ -69528,7 +69543,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>2313</v>
       </c>
@@ -69575,7 +69590,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>2313</v>
       </c>
@@ -69625,7 +69640,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>2313</v>
       </c>
@@ -69675,7 +69690,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>2313</v>
       </c>
@@ -69722,7 +69737,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>2313</v>
       </c>
@@ -69769,7 +69784,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>2313</v>
       </c>
@@ -69816,7 +69831,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>2313</v>
       </c>
@@ -69863,7 +69878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>2313</v>
       </c>
@@ -69910,7 +69925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>2313</v>
       </c>
@@ -69957,7 +69972,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>2313</v>
       </c>
@@ -70005,7 +70020,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>2313</v>
       </c>
@@ -70053,7 +70068,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>2313</v>
       </c>
@@ -70100,7 +70115,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>2313</v>
       </c>
@@ -70147,7 +70162,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>2313</v>
       </c>
@@ -70194,7 +70209,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>2313</v>
       </c>
@@ -70241,7 +70256,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>2313</v>
       </c>
@@ -70288,7 +70303,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>2313</v>
       </c>
@@ -70335,7 +70350,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>2313</v>
       </c>
@@ -70382,7 +70397,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>2313</v>
       </c>
@@ -70429,7 +70444,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>2313</v>
       </c>
@@ -70476,7 +70491,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>2313</v>
       </c>
@@ -70523,7 +70538,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>2313</v>
       </c>
@@ -70570,7 +70585,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>2313</v>
       </c>
@@ -70617,7 +70632,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>2313</v>
       </c>
@@ -70664,7 +70679,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>2313</v>
       </c>
@@ -70711,7 +70726,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>2313</v>
       </c>
@@ -70758,7 +70773,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>2313</v>
       </c>
@@ -70805,7 +70820,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>2313</v>
       </c>
@@ -70855,7 +70870,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>2313</v>
       </c>
@@ -70902,7 +70917,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>2313</v>
       </c>
@@ -70949,7 +70964,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>2313</v>
       </c>
@@ -70996,7 +71011,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>2313</v>
       </c>
@@ -71043,7 +71058,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>2313</v>
       </c>
@@ -71090,7 +71105,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>2313</v>
       </c>
@@ -71137,7 +71152,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>2313</v>
       </c>
@@ -71184,7 +71199,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>2313</v>
       </c>
@@ -71231,7 +71246,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>2313</v>
       </c>
@@ -71278,7 +71293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>2313</v>
       </c>
@@ -71325,7 +71340,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>2313</v>
       </c>
@@ -71372,7 +71387,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>2313</v>
       </c>
@@ -71419,7 +71434,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>2313</v>
       </c>
@@ -71466,7 +71481,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>2313</v>
       </c>
@@ -71513,7 +71528,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>2313</v>
       </c>
@@ -71560,7 +71575,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>2313</v>
       </c>
@@ -71610,7 +71625,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>2313</v>
       </c>
@@ -71657,7 +71672,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>2313</v>
       </c>
@@ -71707,7 +71722,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>2313</v>
       </c>
@@ -71754,7 +71769,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>2313</v>
       </c>
@@ -71804,7 +71819,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>2313</v>
       </c>
@@ -71851,7 +71866,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A129" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71898,7 +71913,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A130" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71945,7 +71960,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2313</v>
       </c>
@@ -71992,7 +72007,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>2313</v>
       </c>
@@ -72039,7 +72054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>2313</v>
       </c>
@@ -72086,7 +72101,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>2313</v>
       </c>
@@ -72133,7 +72148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>2313</v>
       </c>
@@ -72180,7 +72195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>2313</v>
       </c>
@@ -72230,7 +72245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>2313</v>
       </c>
@@ -72277,7 +72292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A138" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72324,7 +72339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>2313</v>
       </c>
@@ -72371,7 +72386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>2313</v>
       </c>
@@ -72418,7 +72433,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>2313</v>
       </c>
@@ -72465,7 +72480,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>2313</v>
       </c>
@@ -72512,7 +72527,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>2313</v>
       </c>
@@ -72559,7 +72574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>2313</v>
       </c>
@@ -72606,7 +72621,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>2313</v>
       </c>
@@ -72653,7 +72668,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>2313</v>
       </c>
@@ -72700,7 +72715,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A147" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72747,7 +72762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A148" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72794,7 +72809,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>2313</v>
       </c>
@@ -72841,7 +72856,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>2313</v>
       </c>
@@ -72888,7 +72903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>2313</v>
       </c>
@@ -72935,7 +72950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>2313</v>
       </c>
@@ -72985,7 +73000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>2313</v>
       </c>
@@ -73032,7 +73047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>2313</v>
       </c>
@@ -73079,7 +73094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A155" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73126,7 +73141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>2313</v>
       </c>
@@ -73173,7 +73188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>2313</v>
       </c>
@@ -73220,7 +73235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>2313</v>
       </c>
@@ -73267,7 +73282,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>2313</v>
       </c>
@@ -73314,7 +73329,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>2313</v>
       </c>
@@ -73361,7 +73376,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>2313</v>
       </c>
@@ -73408,7 +73423,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>2313</v>
       </c>
@@ -73455,7 +73470,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>2313</v>
       </c>
@@ -73502,7 +73517,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>2313</v>
       </c>
@@ -73549,7 +73564,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A165" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73596,7 +73611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A166" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73643,7 +73658,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>2313</v>
       </c>
@@ -73690,7 +73705,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>2313</v>
       </c>
@@ -73737,7 +73752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>2313</v>
       </c>
@@ -73784,7 +73799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>2313</v>
       </c>
@@ -73831,7 +73846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A171" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73878,7 +73893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>2313</v>
       </c>
@@ -73925,7 +73940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>2313</v>
       </c>
@@ -73975,7 +73990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>2313</v>
       </c>
@@ -74022,7 +74037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>2313</v>
       </c>
@@ -74069,7 +74084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>2313</v>
       </c>
@@ -74116,7 +74131,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>2313</v>
       </c>
@@ -74163,7 +74178,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>2313</v>
       </c>
@@ -74210,7 +74225,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>2313</v>
       </c>
@@ -74257,7 +74272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>2313</v>
       </c>
@@ -74304,7 +74319,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>2313</v>
       </c>
@@ -74351,7 +74366,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>2313</v>
       </c>
@@ -74398,7 +74413,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="183" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A183" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74445,7 +74460,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A184" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74492,7 +74507,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>2313</v>
       </c>
@@ -74539,7 +74554,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>2313</v>
       </c>
@@ -74586,7 +74601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>2313</v>
       </c>
@@ -74633,7 +74648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>2313</v>
       </c>
@@ -74680,7 +74695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>2313</v>
       </c>
@@ -74730,7 +74745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>2313</v>
       </c>
@@ -74777,7 +74792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A191" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74824,7 +74839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>2313</v>
       </c>
@@ -74871,7 +74886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>2313</v>
       </c>
@@ -74918,7 +74933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>2313</v>
       </c>
@@ -74965,7 +74980,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>2313</v>
       </c>
@@ -75012,7 +75027,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>2313</v>
       </c>
@@ -75059,7 +75074,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>2313</v>
       </c>
@@ -75106,7 +75121,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>2313</v>
       </c>
@@ -75153,7 +75168,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>2313</v>
       </c>
@@ -75200,7 +75215,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>2313</v>
       </c>
@@ -75247,7 +75262,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>2313</v>
       </c>
@@ -75344,7 +75359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="203" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A203" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75391,7 +75406,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="204" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A204" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75438,7 +75453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="205" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A205" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75485,7 +75500,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>2313</v>
       </c>
@@ -75533,7 +75548,7 @@
       </c>
       <c r="P206" s="3"/>
     </row>
-    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>2313</v>
       </c>
@@ -75581,7 +75596,7 @@
       </c>
       <c r="P207" s="3"/>
     </row>
-    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>2313</v>
       </c>
@@ -75629,7 +75644,7 @@
       </c>
       <c r="P208" s="3"/>
     </row>
-    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>2313</v>
       </c>
@@ -75677,7 +75692,7 @@
       </c>
       <c r="P209" s="3"/>
     </row>
-    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>2313</v>
       </c>
@@ -75725,7 +75740,7 @@
       </c>
       <c r="P210" s="3"/>
     </row>
-    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>2313</v>
       </c>
@@ -75773,7 +75788,7 @@
       </c>
       <c r="P211" s="3"/>
     </row>
-    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>2313</v>
       </c>
@@ -75821,7 +75836,7 @@
       </c>
       <c r="P212" s="3"/>
     </row>
-    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>2313</v>
       </c>
@@ -75869,7 +75884,7 @@
       </c>
       <c r="P213" s="3"/>
     </row>
-    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>2313</v>
       </c>
@@ -75917,7 +75932,7 @@
       </c>
       <c r="P214" s="3"/>
     </row>
-    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>2313</v>
       </c>
@@ -75965,7 +75980,7 @@
       </c>
       <c r="P215" s="3"/>
     </row>
-    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>2313</v>
       </c>
@@ -76013,7 +76028,7 @@
       </c>
       <c r="P216" s="3"/>
     </row>
-    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>2313</v>
       </c>
@@ -76060,7 +76075,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>2313</v>
       </c>
@@ -76107,7 +76122,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>2313</v>
       </c>
@@ -76154,7 +76169,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>2313</v>
       </c>
@@ -76201,7 +76216,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>2313</v>
       </c>
@@ -76248,7 +76263,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>2313</v>
       </c>
@@ -76295,7 +76310,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>2313</v>
       </c>
@@ -76389,7 +76404,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>2313</v>
       </c>
@@ -76436,7 +76451,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>2313</v>
       </c>
@@ -76483,7 +76498,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>2313</v>
       </c>
@@ -76530,7 +76545,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>2313</v>
       </c>
@@ -76577,7 +76592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>2313</v>
       </c>
@@ -76624,7 +76639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>2313</v>
       </c>
@@ -76671,7 +76686,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>2313</v>
       </c>
@@ -76718,7 +76733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>2685</v>
       </c>
@@ -76765,7 +76780,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>2654</v>
       </c>
@@ -76810,7 +76825,7 @@
       </c>
       <c r="P233" s="3"/>
     </row>
-    <row r="234" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>2313</v>
       </c>
@@ -76857,7 +76872,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>2685</v>
       </c>
@@ -76904,7 +76919,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>2685</v>
       </c>
@@ -76951,7 +76966,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>2685</v>
       </c>
@@ -76998,7 +77013,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>2685</v>
       </c>
@@ -77045,7 +77060,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>2685</v>
       </c>
@@ -77092,7 +77107,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>2685</v>
       </c>
@@ -77139,7 +77154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>2685</v>
       </c>
@@ -77233,7 +77248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>2313</v>
       </c>
@@ -77280,7 +77295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>2313</v>
       </c>
@@ -77327,7 +77342,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>2313</v>
       </c>
@@ -77374,7 +77389,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>2313</v>
       </c>
@@ -77421,7 +77436,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>2313</v>
       </c>
@@ -77468,7 +77483,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>2313</v>
       </c>
@@ -77562,7 +77577,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>2313</v>
       </c>
@@ -77609,7 +77624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>2313</v>
       </c>
@@ -77656,7 +77671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>2313</v>
       </c>
@@ -77703,7 +77718,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>2313</v>
       </c>
@@ -77797,7 +77812,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>2313</v>
       </c>
@@ -77844,7 +77859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>2313</v>
       </c>
@@ -77891,7 +77906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>2313</v>
       </c>
@@ -77938,7 +77953,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="258" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A258" s="13" t="s">
         <v>2313</v>
       </c>
@@ -78032,7 +78047,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2313</v>
       </c>
@@ -78079,7 +78094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2313</v>
       </c>
@@ -78126,7 +78141,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2313</v>
       </c>
@@ -78173,7 +78188,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2313</v>
       </c>
@@ -78220,7 +78235,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2313</v>
       </c>
@@ -78267,7 +78282,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2313</v>
       </c>
@@ -78314,7 +78329,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A266" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78361,7 +78376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A267" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78408,7 +78423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A268" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78455,7 +78470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A269" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78502,7 +78517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A270" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78596,7 +78611,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A272" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78637,7 +78652,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="273" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A273" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78678,7 +78693,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="274" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A274" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78725,7 +78740,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A275" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78772,7 +78787,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="276" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A276" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78819,7 +78834,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A277" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78863,7 +78878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A278" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78910,7 +78925,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>2313</v>
       </c>
@@ -78957,7 +78972,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>2313</v>
       </c>
@@ -79004,7 +79019,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>2313</v>
       </c>
@@ -79051,7 +79066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>2313</v>
       </c>
@@ -79098,7 +79113,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="283" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>2313</v>
       </c>
@@ -79145,7 +79160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>2313</v>
       </c>
@@ -79192,7 +79207,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>2313</v>
       </c>
@@ -79239,7 +79254,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>2313</v>
       </c>
@@ -79286,7 +79301,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>2313</v>
       </c>
@@ -79333,7 +79348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>2313</v>
       </c>
@@ -79380,7 +79395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>2313</v>
       </c>
@@ -79427,7 +79442,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="290" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>2313</v>
       </c>
@@ -79474,7 +79489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="291" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>2313</v>
       </c>
@@ -79521,7 +79536,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="292" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>2313</v>
       </c>
@@ -79568,7 +79583,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="293" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>2313</v>
       </c>
@@ -79615,7 +79630,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="294" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>2313</v>
       </c>
@@ -79662,7 +79677,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="295" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>2313</v>
       </c>
@@ -79709,7 +79724,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="296" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>2313</v>
       </c>
@@ -79756,7 +79771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>2313</v>
       </c>
@@ -79803,7 +79818,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>2313</v>
       </c>
@@ -79850,7 +79865,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="299" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>2313</v>
       </c>
@@ -79897,7 +79912,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="300" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>2313</v>
       </c>
@@ -79944,7 +79959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>2313</v>
       </c>
@@ -79991,7 +80006,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="302" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>2313</v>
       </c>
@@ -80038,7 +80053,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2313</v>
       </c>
@@ -80085,7 +80100,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2313</v>
       </c>
@@ -80132,7 +80147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2313</v>
       </c>
@@ -80179,7 +80194,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2313</v>
       </c>
@@ -80226,7 +80241,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2313</v>
       </c>
@@ -80273,7 +80288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="308" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2313</v>
       </c>
@@ -80320,32 +80335,56 @@
         <v>7</v>
       </c>
     </row>
+    <row r="309" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A309" s="33" t="s">
+        <v>2313</v>
+      </c>
+      <c r="B309" s="33" t="s">
+        <v>664</v>
+      </c>
+      <c r="C309" s="33" t="s">
+        <v>2314</v>
+      </c>
+      <c r="D309" s="33" t="s">
+        <v>2912</v>
+      </c>
+      <c r="E309" s="37" t="s">
+        <v>2852</v>
+      </c>
+      <c r="F309" s="37" t="s">
+        <v>2852</v>
+      </c>
+      <c r="G309" s="33" t="s">
+        <v>2317</v>
+      </c>
+      <c r="H309" s="33" t="s">
+        <v>2318</v>
+      </c>
+      <c r="I309" s="33" t="s">
+        <v>2499</v>
+      </c>
+      <c r="J309" s="37" t="s">
+        <v>2852</v>
+      </c>
+      <c r="K309" s="33" t="s">
+        <v>2499</v>
+      </c>
+      <c r="L309" s="36" t="s">
+        <v>2857</v>
+      </c>
+      <c r="M309" s="37" t="s">
+        <v>2853</v>
+      </c>
+      <c r="N309" s="33"/>
+      <c r="O309" s="35" t="s">
+        <v>2321</v>
+      </c>
+      <c r="P309" s="34">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="1000AC0520"/>
-        <filter val="1000AC4501"/>
-        <filter val="1000AC4502"/>
-        <filter val="1000AC4503"/>
-        <filter val="1000AC4505"/>
-        <filter val="1000AC4507"/>
-        <filter val="1000AC4508"/>
-        <filter val="1001AD0506"/>
-        <filter val="1001AD4527"/>
-        <filter val="1001AD4540"/>
-        <filter val="1002AD0507"/>
-        <filter val="1003AD0507"/>
-        <filter val="1003AD4500"/>
-        <filter val="1005AD0508"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="9">
-      <filters>
-        <filter val="VP Asuntos Corporativos"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P308" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}"/>
   <conditionalFormatting sqref="D278 D1:D271">
     <cfRule type="duplicateValues" dxfId="10" priority="1"/>
     <cfRule type="duplicateValues" dxfId="9" priority="11"/>
@@ -80398,6 +80437,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100CAB26C5234A12E419316CB59C6D7D393" ma:contentTypeVersion="19" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="397be35540538177477362f87776d70c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36cf8265-5d49-4303-8d6c-a3e3dc13898a" xmlns:ns3="70b3a8a4-10f1-4453-b557-059c8aa2e01d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1417ff6b849ed53f32fc8c47614195ac" ns2:_="" ns3:_="">
     <xsd:import namespace="36cf8265-5d49-4303-8d6c-a3e3dc13898a"/>
@@ -80658,15 +80706,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CF387E-488B-4455-A180-73B07596DA96}">
   <ds:schemaRefs>
@@ -80679,6 +80718,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2985AAD5-32B5-43F0-8227-A4AC877DE8D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -80695,12 +80742,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C28E532-0D32-468D-9BC3-E75FD228039A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ajustes manuales para forecast, corrección dif
</commit_message>
<xml_diff>
--- a/v2/uploads/diccionario/CECOS.xlsx
+++ b/v2/uploads/diccionario/CECOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsmmadrida\Repositorios Personales Control Gestion\amsa-budget-corporativo\v2\uploads\diccionario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A5FB96D-7F00-4DC2-BDF7-36469A571598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A177C129-0134-4C3B-AA4F-FF1BB4D613D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{26AC6B6C-E551-4F84-9810-86049090F8FC}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <definedName name="__FPMExcelClient_Connection" localSheetId="2">"_FPM_BPCNW10_[http://10.87.9.254:8000/sap/bpc/]_[PPTO_AMSA]_[AMSA_PARAMETROS]_[false]_[false]\1"</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CECOS Compañías'!$A$1:$N$943</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CECOS Corporativo'!$A$1:$P$280</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CECOS Corporativo Nueva'!$A$1:$P$309</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CECOS Corporativo Nueva'!$A$1:$P$310</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -9560,27 +9560,7 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="22">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -65764,35 +65744,35 @@
   </sheetData>
   <autoFilter ref="A1:P280" xr:uid="{0F1984F8-98C5-4A25-A41F-F7A74C418877}"/>
   <conditionalFormatting sqref="D1:D273 D280">
-    <cfRule type="duplicateValues" dxfId="23" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I251">
-    <cfRule type="duplicateValues" dxfId="21" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I254">
-    <cfRule type="duplicateValues" dxfId="20" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I256">
-    <cfRule type="duplicateValues" dxfId="19" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K251">
-    <cfRule type="duplicateValues" dxfId="18" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K254">
-    <cfRule type="duplicateValues" dxfId="17" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K256">
-    <cfRule type="duplicateValues" dxfId="16" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K261">
-    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K264">
-    <cfRule type="duplicateValues" dxfId="14" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K266">
-    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -65804,7 +65784,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:P310"/>
@@ -65924,7 +65904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2313</v>
       </c>
@@ -66018,7 +65998,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2313</v>
       </c>
@@ -66065,7 +66045,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2313</v>
       </c>
@@ -66112,7 +66092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2313</v>
       </c>
@@ -66159,7 +66139,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2313</v>
       </c>
@@ -66206,7 +66186,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2313</v>
       </c>
@@ -66253,7 +66233,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2313</v>
       </c>
@@ -66300,7 +66280,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2313</v>
       </c>
@@ -66347,7 +66327,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>2313</v>
       </c>
@@ -66397,7 +66377,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2313</v>
       </c>
@@ -66445,7 +66425,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>2313</v>
       </c>
@@ -66492,7 +66472,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2313</v>
       </c>
@@ -66539,7 +66519,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>2313</v>
       </c>
@@ -66586,7 +66566,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2313</v>
       </c>
@@ -66633,7 +66613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2313</v>
       </c>
@@ -66680,7 +66660,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>2313</v>
       </c>
@@ -66727,7 +66707,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2313</v>
       </c>
@@ -66774,7 +66754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>2313</v>
       </c>
@@ -66824,7 +66804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>2313</v>
       </c>
@@ -66871,7 +66851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2313</v>
       </c>
@@ -66918,7 +66898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2313</v>
       </c>
@@ -66965,7 +66945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2313</v>
       </c>
@@ -67012,7 +66992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2313</v>
       </c>
@@ -67059,7 +67039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>2313</v>
       </c>
@@ -67106,7 +67086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2313</v>
       </c>
@@ -67156,7 +67136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2313</v>
       </c>
@@ -67203,7 +67183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2313</v>
       </c>
@@ -67250,7 +67230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>2313</v>
       </c>
@@ -67297,7 +67277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2313</v>
       </c>
@@ -67347,7 +67327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2313</v>
       </c>
@@ -67394,7 +67374,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>2313</v>
       </c>
@@ -67441,7 +67421,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>2313</v>
       </c>
@@ -67488,7 +67468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>2313</v>
       </c>
@@ -67535,7 +67515,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>2313</v>
       </c>
@@ -67582,7 +67562,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>2313</v>
       </c>
@@ -67629,7 +67609,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>2313</v>
       </c>
@@ -67676,7 +67656,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>2313</v>
       </c>
@@ -67723,7 +67703,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>2313</v>
       </c>
@@ -67770,7 +67750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>2313</v>
       </c>
@@ -67817,7 +67797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>2313</v>
       </c>
@@ -67864,7 +67844,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>2313</v>
       </c>
@@ -67911,7 +67891,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>2313</v>
       </c>
@@ -67958,7 +67938,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>2313</v>
       </c>
@@ -68005,7 +67985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>2313</v>
       </c>
@@ -68052,7 +68032,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>2313</v>
       </c>
@@ -68099,7 +68079,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>2313</v>
       </c>
@@ -68149,7 +68129,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>2313</v>
       </c>
@@ -68199,7 +68179,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>2313</v>
       </c>
@@ -68246,7 +68226,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>2313</v>
       </c>
@@ -68293,7 +68273,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>2313</v>
       </c>
@@ -68340,7 +68320,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>2313</v>
       </c>
@@ -68387,7 +68367,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>2313</v>
       </c>
@@ -68434,7 +68414,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>2313</v>
       </c>
@@ -68481,7 +68461,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>2313</v>
       </c>
@@ -68528,7 +68508,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>2313</v>
       </c>
@@ -68575,7 +68555,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>2313</v>
       </c>
@@ -68622,7 +68602,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>2313</v>
       </c>
@@ -68669,7 +68649,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>2313</v>
       </c>
@@ -68716,7 +68696,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>2313</v>
       </c>
@@ -68763,7 +68743,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>2313</v>
       </c>
@@ -68810,7 +68790,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>2313</v>
       </c>
@@ -68857,7 +68837,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>2313</v>
       </c>
@@ -68904,7 +68884,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>2313</v>
       </c>
@@ -68951,7 +68931,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>2313</v>
       </c>
@@ -69001,7 +68981,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>2313</v>
       </c>
@@ -69048,7 +69028,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>2313</v>
       </c>
@@ -69095,7 +69075,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>2313</v>
       </c>
@@ -69142,7 +69122,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>2313</v>
       </c>
@@ -69192,7 +69172,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>2313</v>
       </c>
@@ -69239,7 +69219,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>2313</v>
       </c>
@@ -69286,7 +69266,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>2313</v>
       </c>
@@ -69336,7 +69316,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>2313</v>
       </c>
@@ -69384,7 +69364,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>2313</v>
       </c>
@@ -69431,7 +69411,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>2313</v>
       </c>
@@ -69481,7 +69461,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>2313</v>
       </c>
@@ -69528,7 +69508,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>2313</v>
       </c>
@@ -69575,7 +69555,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>2313</v>
       </c>
@@ -69622,7 +69602,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>2313</v>
       </c>
@@ -69672,7 +69652,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>2313</v>
       </c>
@@ -69722,7 +69702,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>2313</v>
       </c>
@@ -69769,7 +69749,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>2313</v>
       </c>
@@ -69816,7 +69796,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>2313</v>
       </c>
@@ -69863,7 +69843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>2313</v>
       </c>
@@ -69910,7 +69890,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>2313</v>
       </c>
@@ -69957,7 +69937,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>2313</v>
       </c>
@@ -70004,7 +69984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>2313</v>
       </c>
@@ -70052,7 +70032,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>2313</v>
       </c>
@@ -70100,7 +70080,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>2313</v>
       </c>
@@ -70147,7 +70127,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>2313</v>
       </c>
@@ -70194,7 +70174,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>2313</v>
       </c>
@@ -70241,7 +70221,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>2313</v>
       </c>
@@ -70288,7 +70268,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>2313</v>
       </c>
@@ -70335,7 +70315,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>2313</v>
       </c>
@@ -70382,7 +70362,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>2313</v>
       </c>
@@ -70429,7 +70409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>2313</v>
       </c>
@@ -70476,7 +70456,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>2313</v>
       </c>
@@ -70523,7 +70503,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>2313</v>
       </c>
@@ -70570,7 +70550,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>2313</v>
       </c>
@@ -70617,7 +70597,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>2313</v>
       </c>
@@ -70664,7 +70644,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>2313</v>
       </c>
@@ -70711,7 +70691,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>2313</v>
       </c>
@@ -70758,7 +70738,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>2313</v>
       </c>
@@ -70805,7 +70785,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>2313</v>
       </c>
@@ -70852,7 +70832,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>2313</v>
       </c>
@@ -70902,7 +70882,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>2313</v>
       </c>
@@ -70949,7 +70929,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>2313</v>
       </c>
@@ -70996,7 +70976,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>2313</v>
       </c>
@@ -71043,7 +71023,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>2313</v>
       </c>
@@ -71090,7 +71070,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>2313</v>
       </c>
@@ -71137,7 +71117,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>2313</v>
       </c>
@@ -71184,7 +71164,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>2313</v>
       </c>
@@ -71231,7 +71211,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>2313</v>
       </c>
@@ -71278,7 +71258,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>2313</v>
       </c>
@@ -71325,7 +71305,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>2313</v>
       </c>
@@ -71372,7 +71352,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>2313</v>
       </c>
@@ -71419,7 +71399,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>2313</v>
       </c>
@@ -71466,7 +71446,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>2313</v>
       </c>
@@ -71513,7 +71493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>2313</v>
       </c>
@@ -71560,7 +71540,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>2313</v>
       </c>
@@ -71607,7 +71587,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>2313</v>
       </c>
@@ -71657,7 +71637,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>2313</v>
       </c>
@@ -71704,7 +71684,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>2313</v>
       </c>
@@ -71754,7 +71734,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>2313</v>
       </c>
@@ -71801,7 +71781,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>2313</v>
       </c>
@@ -71851,7 +71831,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>2313</v>
       </c>
@@ -71945,7 +71925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A130" s="27" t="s">
         <v>2313</v>
       </c>
@@ -71992,7 +71972,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2313</v>
       </c>
@@ -72039,7 +72019,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>2313</v>
       </c>
@@ -72086,7 +72066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>2313</v>
       </c>
@@ -72133,7 +72113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>2313</v>
       </c>
@@ -72180,7 +72160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>2313</v>
       </c>
@@ -72227,7 +72207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>2313</v>
       </c>
@@ -72277,7 +72257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>2313</v>
       </c>
@@ -72324,7 +72304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A138" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72371,7 +72351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>2313</v>
       </c>
@@ -72418,7 +72398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>2313</v>
       </c>
@@ -72465,7 +72445,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>2313</v>
       </c>
@@ -72512,7 +72492,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>2313</v>
       </c>
@@ -72559,7 +72539,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>2313</v>
       </c>
@@ -72606,7 +72586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>2313</v>
       </c>
@@ -72653,7 +72633,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>2313</v>
       </c>
@@ -72700,7 +72680,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>2313</v>
       </c>
@@ -72794,7 +72774,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A148" s="27" t="s">
         <v>2313</v>
       </c>
@@ -72841,7 +72821,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>2313</v>
       </c>
@@ -72888,7 +72868,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>2313</v>
       </c>
@@ -72935,7 +72915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>2313</v>
       </c>
@@ -72982,7 +72962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>2313</v>
       </c>
@@ -73032,7 +73012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>2313</v>
       </c>
@@ -73079,7 +73059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>2313</v>
       </c>
@@ -73126,7 +73106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A155" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73173,7 +73153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>2313</v>
       </c>
@@ -73220,7 +73200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>2313</v>
       </c>
@@ -73267,7 +73247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>2313</v>
       </c>
@@ -73314,7 +73294,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>2313</v>
       </c>
@@ -73361,7 +73341,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>2313</v>
       </c>
@@ -73408,7 +73388,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>2313</v>
       </c>
@@ -73455,7 +73435,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>2313</v>
       </c>
@@ -73502,7 +73482,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>2313</v>
       </c>
@@ -73549,7 +73529,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>2313</v>
       </c>
@@ -73643,7 +73623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A166" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73690,7 +73670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>2313</v>
       </c>
@@ -73737,7 +73717,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>2313</v>
       </c>
@@ -73784,7 +73764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>2313</v>
       </c>
@@ -73831,7 +73811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>2313</v>
       </c>
@@ -73878,7 +73858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A171" s="27" t="s">
         <v>2313</v>
       </c>
@@ -73925,7 +73905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>2313</v>
       </c>
@@ -73972,7 +73952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>2313</v>
       </c>
@@ -74022,7 +74002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>2313</v>
       </c>
@@ -74069,7 +74049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>2313</v>
       </c>
@@ -74116,7 +74096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>2313</v>
       </c>
@@ -74163,7 +74143,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>2313</v>
       </c>
@@ -74210,7 +74190,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>2313</v>
       </c>
@@ -74257,7 +74237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>2313</v>
       </c>
@@ -74304,7 +74284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>2313</v>
       </c>
@@ -74351,7 +74331,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>2313</v>
       </c>
@@ -74398,7 +74378,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>2313</v>
       </c>
@@ -74492,7 +74472,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A184" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74539,7 +74519,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>2313</v>
       </c>
@@ -74586,7 +74566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>2313</v>
       </c>
@@ -74633,7 +74613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>2313</v>
       </c>
@@ -74680,7 +74660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>2313</v>
       </c>
@@ -74727,7 +74707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>2313</v>
       </c>
@@ -74777,7 +74757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>2313</v>
       </c>
@@ -74824,7 +74804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A191" s="27" t="s">
         <v>2313</v>
       </c>
@@ -74871,7 +74851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>2313</v>
       </c>
@@ -74918,7 +74898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>2313</v>
       </c>
@@ -74965,7 +74945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>2313</v>
       </c>
@@ -75012,7 +74992,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>2313</v>
       </c>
@@ -75059,7 +75039,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>2313</v>
       </c>
@@ -75106,7 +75086,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>2313</v>
       </c>
@@ -75153,7 +75133,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>2313</v>
       </c>
@@ -75200,7 +75180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>2313</v>
       </c>
@@ -75247,7 +75227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>2313</v>
       </c>
@@ -75294,7 +75274,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>2313</v>
       </c>
@@ -75341,7 +75321,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>2313</v>
       </c>
@@ -75391,7 +75371,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="203" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A203" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75438,7 +75418,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="204" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A204" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75485,7 +75465,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="205" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A205" s="13" t="s">
         <v>2313</v>
       </c>
@@ -75532,7 +75512,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>2313</v>
       </c>
@@ -75580,7 +75560,7 @@
       </c>
       <c r="P206" s="3"/>
     </row>
-    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>2313</v>
       </c>
@@ -75628,7 +75608,7 @@
       </c>
       <c r="P207" s="3"/>
     </row>
-    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>2313</v>
       </c>
@@ -75676,7 +75656,7 @@
       </c>
       <c r="P208" s="3"/>
     </row>
-    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>2313</v>
       </c>
@@ -75724,7 +75704,7 @@
       </c>
       <c r="P209" s="3"/>
     </row>
-    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>2313</v>
       </c>
@@ -75772,7 +75752,7 @@
       </c>
       <c r="P210" s="3"/>
     </row>
-    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>2313</v>
       </c>
@@ -75820,7 +75800,7 @@
       </c>
       <c r="P211" s="3"/>
     </row>
-    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>2313</v>
       </c>
@@ -75868,7 +75848,7 @@
       </c>
       <c r="P212" s="3"/>
     </row>
-    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>2313</v>
       </c>
@@ -75916,7 +75896,7 @@
       </c>
       <c r="P213" s="3"/>
     </row>
-    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>2313</v>
       </c>
@@ -75964,7 +75944,7 @@
       </c>
       <c r="P214" s="3"/>
     </row>
-    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>2313</v>
       </c>
@@ -76012,7 +75992,7 @@
       </c>
       <c r="P215" s="3"/>
     </row>
-    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>2313</v>
       </c>
@@ -76060,7 +76040,7 @@
       </c>
       <c r="P216" s="3"/>
     </row>
-    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>2313</v>
       </c>
@@ -76107,7 +76087,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>2313</v>
       </c>
@@ -76154,7 +76134,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>2313</v>
       </c>
@@ -76201,7 +76181,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>2313</v>
       </c>
@@ -76248,7 +76228,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>2313</v>
       </c>
@@ -76295,7 +76275,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>2313</v>
       </c>
@@ -76342,7 +76322,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>2313</v>
       </c>
@@ -76389,7 +76369,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>2313</v>
       </c>
@@ -76436,7 +76416,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>2313</v>
       </c>
@@ -76483,7 +76463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>2313</v>
       </c>
@@ -76530,7 +76510,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>2313</v>
       </c>
@@ -76577,7 +76557,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>2313</v>
       </c>
@@ -76624,7 +76604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>2313</v>
       </c>
@@ -76671,7 +76651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>2313</v>
       </c>
@@ -76718,7 +76698,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>2313</v>
       </c>
@@ -76765,7 +76745,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>2685</v>
       </c>
@@ -76812,7 +76792,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>2654</v>
       </c>
@@ -76857,7 +76837,7 @@
       </c>
       <c r="P233" s="3"/>
     </row>
-    <row r="234" spans="1:16" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>2313</v>
       </c>
@@ -76904,7 +76884,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>2685</v>
       </c>
@@ -76951,7 +76931,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>2685</v>
       </c>
@@ -76998,7 +76978,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>2685</v>
       </c>
@@ -77045,7 +77025,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>2685</v>
       </c>
@@ -77092,7 +77072,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>2685</v>
       </c>
@@ -77139,7 +77119,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>2685</v>
       </c>
@@ -77186,7 +77166,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>2685</v>
       </c>
@@ -77233,7 +77213,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>2313</v>
       </c>
@@ -77280,7 +77260,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>2313</v>
       </c>
@@ -77327,7 +77307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>2313</v>
       </c>
@@ -77374,7 +77354,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>2313</v>
       </c>
@@ -77421,7 +77401,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>2313</v>
       </c>
@@ -77468,7 +77448,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>2313</v>
       </c>
@@ -77515,7 +77495,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>2313</v>
       </c>
@@ -77562,7 +77542,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>2313</v>
       </c>
@@ -77609,7 +77589,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>2313</v>
       </c>
@@ -77656,7 +77636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>2313</v>
       </c>
@@ -77703,7 +77683,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>2313</v>
       </c>
@@ -77750,7 +77730,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>2313</v>
       </c>
@@ -77797,7 +77777,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>2313</v>
       </c>
@@ -77844,7 +77824,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>2313</v>
       </c>
@@ -77891,7 +77871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>2313</v>
       </c>
@@ -77938,7 +77918,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>2313</v>
       </c>
@@ -77985,7 +77965,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="258" spans="1:16" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A258" s="13" t="s">
         <v>2313</v>
       </c>
@@ -78032,7 +78012,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2313</v>
       </c>
@@ -78079,7 +78059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2313</v>
       </c>
@@ -78126,7 +78106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2313</v>
       </c>
@@ -78173,7 +78153,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2313</v>
       </c>
@@ -78220,7 +78200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2313</v>
       </c>
@@ -78267,7 +78247,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2313</v>
       </c>
@@ -78314,7 +78294,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2313</v>
       </c>
@@ -78361,7 +78341,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A266" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78408,7 +78388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A267" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78455,7 +78435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A268" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78502,7 +78482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:16" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:16" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A269" s="29" t="s">
         <v>2313</v>
       </c>
@@ -78596,7 +78576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A271" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78643,7 +78623,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A272" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78684,7 +78664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="273" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A273" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78725,7 +78705,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="274" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A274" s="11" t="s">
         <v>2685</v>
       </c>
@@ -78772,7 +78752,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A275" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78800,8 +78780,8 @@
       <c r="I275" s="11" t="s">
         <v>2836</v>
       </c>
-      <c r="J275" s="11" t="s">
-        <v>2833</v>
+      <c r="J275" t="s">
+        <v>2699</v>
       </c>
       <c r="K275" s="11" t="s">
         <v>2836</v>
@@ -78819,7 +78799,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="276" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A276" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78847,8 +78827,8 @@
       <c r="I276" s="11" t="s">
         <v>2841</v>
       </c>
-      <c r="J276" s="11" t="s">
-        <v>2838</v>
+      <c r="J276" t="s">
+        <v>2699</v>
       </c>
       <c r="K276" s="11" t="s">
         <v>2841</v>
@@ -78866,7 +78846,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A277" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78910,7 +78890,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:16" s="11" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A278" s="11" t="s">
         <v>2313</v>
       </c>
@@ -78957,7 +78937,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>2313</v>
       </c>
@@ -79004,7 +78984,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>2313</v>
       </c>
@@ -79051,7 +79031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>2313</v>
       </c>
@@ -79098,7 +79078,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>2313</v>
       </c>
@@ -79145,7 +79125,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="283" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>2313</v>
       </c>
@@ -79192,7 +79172,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>2313</v>
       </c>
@@ -79239,7 +79219,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>2313</v>
       </c>
@@ -79286,7 +79266,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>2313</v>
       </c>
@@ -79333,7 +79313,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>2313</v>
       </c>
@@ -79380,7 +79360,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>2313</v>
       </c>
@@ -79427,7 +79407,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>2313</v>
       </c>
@@ -79474,7 +79454,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="290" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>2313</v>
       </c>
@@ -79521,7 +79501,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="291" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>2313</v>
       </c>
@@ -79568,7 +79548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="292" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>2313</v>
       </c>
@@ -79615,7 +79595,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="293" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>2313</v>
       </c>
@@ -79662,7 +79642,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="294" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>2313</v>
       </c>
@@ -79709,7 +79689,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="295" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>2313</v>
       </c>
@@ -79756,7 +79736,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="296" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>2313</v>
       </c>
@@ -79803,7 +79783,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>2313</v>
       </c>
@@ -79850,7 +79830,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>2313</v>
       </c>
@@ -79897,7 +79877,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="299" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>2313</v>
       </c>
@@ -79944,7 +79924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="300" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>2313</v>
       </c>
@@ -79991,7 +79971,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>2313</v>
       </c>
@@ -80038,7 +80018,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="302" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>2313</v>
       </c>
@@ -80085,7 +80065,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2313</v>
       </c>
@@ -80132,7 +80112,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2313</v>
       </c>
@@ -80179,7 +80159,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2313</v>
       </c>
@@ -80226,7 +80206,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2313</v>
       </c>
@@ -80273,7 +80253,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2313</v>
       </c>
@@ -80320,7 +80300,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="308" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2313</v>
       </c>
@@ -80367,7 +80347,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="309" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>2313</v>
       </c>
@@ -80462,43 +80442,37 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P309" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="VP Exploraciones y Recursos Mineros"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P310" xr:uid="{2DAE5BBC-D8BD-4F3A-9CAD-E145EDF81891}"/>
   <conditionalFormatting sqref="D278 D1:D271">
-    <cfRule type="duplicateValues" dxfId="12" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I249">
-    <cfRule type="duplicateValues" dxfId="10" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I252">
-    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I254">
-    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K249">
-    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K252">
-    <cfRule type="duplicateValues" dxfId="6" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K254">
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K259">
-    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K262">
-    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K264">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>